<commit_message>
feat: importar 50 lojas da shopee via csv
</commit_message>
<xml_diff>
--- a/shopee.xlsx
+++ b/shopee.xlsx
@@ -397,15 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="50.83203125" customWidth="1"/>
-    <col min="3" max="3" width="40.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:F51"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,67 +421,1007 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kit 3 Cremes Nativa Spa</v>
+        <v>LAA COSMÉTICOS</v>
       </c>
       <c r="B2" t="str">
-        <v>Hidratação profunda e fragrância irresistível.</v>
+        <v>Loja em Destaque - Até 83%</v>
       </c>
       <c r="C2" t="str">
-        <v>https://shopee.com.br/product/1420372901/58202126334</v>
+        <v>https://s.shopee.com.br/50VUBBBJ56</v>
       </c>
       <c r="D2" t="str">
-        <v>sparkles</v>
+        <v>shopping-bag</v>
       </c>
       <c r="E2" t="str">
-        <v>#ee4d2d</v>
+        <v>#f53d2d</v>
       </c>
       <c r="F2" t="str">
-        <v>🔥 Top 1</v>
+        <v>Top Loja</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Shampoo Tonalizante Matizze</v>
+        <v>The Foods</v>
       </c>
       <c r="B3" t="str">
-        <v>Escurecedor natural sem amônia. Resultados rápidos!</v>
+        <v>Loja em Destaque - Até 83%</v>
       </c>
       <c r="C3" t="str">
-        <v>https://shopee.com.br/product/422903557/22994840965</v>
+        <v>https://s.shopee.com.br/5AouNUAfk9</v>
       </c>
       <c r="D3" t="str">
-        <v>scissors</v>
+        <v>shopping-bag</v>
       </c>
       <c r="E3" t="str">
-        <v>#ee4d2d</v>
+        <v>#f53d2d</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>Top Loja</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Projetor HY300 Smart</v>
+        <v>Helô Naturais</v>
       </c>
       <c r="B4" t="str">
-        <v>Cinema em casa com Android 11 e resolução 4K.</v>
+        <v>Loja em Destaque - Até 83%</v>
       </c>
       <c r="C4" t="str">
-        <v>https://shopee.com.br/search?keyword=projetor%20hy300</v>
+        <v>https://s.shopee.com.br/4fsdmZCZl4</v>
       </c>
       <c r="D4" t="str">
-        <v>monitor</v>
+        <v>shopping-bag</v>
       </c>
       <c r="E4" t="str">
-        <v>#ee4d2d</v>
+        <v>#f53d2d</v>
       </c>
       <c r="F4" t="str">
-        <v>⚡ Oferta</v>
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Alfa Colors</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Loja em Destaque - Até 83%</v>
+      </c>
+      <c r="C5" t="str">
+        <v>https://s.shopee.com.br/4qC3ysBwQ7</v>
+      </c>
+      <c r="D5" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E5" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>isabella vendas</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Loja em Destaque - Até 83%</v>
+      </c>
+      <c r="C6" t="str">
+        <v>https://s.shopee.com.br/4LFnNxDqR2</v>
+      </c>
+      <c r="D6" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E6" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>MALUKA MODAS</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Loja em Destaque - Até 83%</v>
+      </c>
+      <c r="C7" t="str">
+        <v>https://s.shopee.com.br/4VZDaGDD65</v>
+      </c>
+      <c r="D7" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E7" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Fruttato</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Loja em Destaque - Até 83%</v>
+      </c>
+      <c r="C8" t="str">
+        <v>https://s.shopee.com.br/40cwzLF770</v>
+      </c>
+      <c r="D8" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E8" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>detecidos</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Loja em Destaque - Até 83%</v>
+      </c>
+      <c r="C9" t="str">
+        <v>https://s.shopee.com.br/4AwNBeETm3</v>
+      </c>
+      <c r="D9" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E9" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Departamento Paulista Store</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Loja em Destaque - Até 83%</v>
+      </c>
+      <c r="C10" t="str">
+        <v>https://s.shopee.com.br/3g06ajGNmy</v>
+      </c>
+      <c r="D10" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E10" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Shop Fácil Store</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Loja em Destaque - Até 82%</v>
+      </c>
+      <c r="C11" t="str">
+        <v>https://s.shopee.com.br/3qJWn2FkS1</v>
+      </c>
+      <c r="D11" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E11" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Mato Grosso Naturais</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Loja em Destaque - Até 82%</v>
+      </c>
+      <c r="C12" t="str">
+        <v>https://s.shopee.com.br/3LNGC7HeSw</v>
+      </c>
+      <c r="D12" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E12" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Apolo Decor</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Loja em Destaque - Até 80%</v>
+      </c>
+      <c r="C13" t="str">
+        <v>https://s.shopee.com.br/3VggOQH17z</v>
+      </c>
+      <c r="D13" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E13" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>* TopVendarj *</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Loja em Destaque - Até 80%</v>
+      </c>
+      <c r="C14" t="str">
+        <v>https://s.shopee.com.br/30kPnVIv8u</v>
+      </c>
+      <c r="D14" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E14" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Comercial SD Eletro-Eletrônico</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Loja em Destaque - Até 78%</v>
+      </c>
+      <c r="C15" t="str">
+        <v>https://s.shopee.com.br/3B3pzoIHnx</v>
+      </c>
+      <c r="D15" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E15" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>FÊNIX FRF</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Loja em Destaque - Até 77%</v>
+      </c>
+      <c r="C16" t="str">
+        <v>https://s.shopee.com.br/2g7ZOtKBos</v>
+      </c>
+      <c r="D16" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E16" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TTL PAINEIS E ARTESANATO</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Loja em Destaque - Até 73%</v>
+      </c>
+      <c r="C17" t="str">
+        <v>https://s.shopee.com.br/2qQzbCJYTv</v>
+      </c>
+      <c r="D17" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E17" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Viking Repelentes</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Loja em Destaque - Até 73%</v>
+      </c>
+      <c r="C18" t="str">
+        <v>https://s.shopee.com.br/2LUj0HLSUq</v>
+      </c>
+      <c r="D18" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E18" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Márcia Cardoso de Oliveira lima</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Loja em Destaque - Até 71%</v>
+      </c>
+      <c r="C19" t="str">
+        <v>https://s.shopee.com.br/2Vo9CaKp9t</v>
+      </c>
+      <c r="D19" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E19" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Tomate Racing33</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Loja em Destaque - Até 69%</v>
+      </c>
+      <c r="C20" t="str">
+        <v>https://s.shopee.com.br/20rsbfMjAo</v>
+      </c>
+      <c r="D20" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E20" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Fernandes_Arts</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Loja em Destaque - Até 68,78%</v>
+      </c>
+      <c r="C21" t="str">
+        <v>https://s.shopee.com.br/2BBInyM5pr</v>
+      </c>
+      <c r="D21" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E21" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Galera Adesivos</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Loja em Destaque - Até 66,78%</v>
+      </c>
+      <c r="C22" t="str">
+        <v>https://s.shopee.com.br/1gF2D3Nzqm</v>
+      </c>
+      <c r="D22" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E22" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>We Curve Estilos</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Loja em Destaque - Até 63%</v>
+      </c>
+      <c r="C23" t="str">
+        <v>https://s.shopee.com.br/1qYSPMNMVp</v>
+      </c>
+      <c r="D23" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E23" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>STD Nutraceuticals</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Loja em Destaque - Até 62%</v>
+      </c>
+      <c r="C24" t="str">
+        <v>https://s.shopee.com.br/1LcBoRPGWk</v>
+      </c>
+      <c r="D24" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E24" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>To Aqui Shop</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Loja em Destaque - Até 62%</v>
+      </c>
+      <c r="C25" t="str">
+        <v>https://s.shopee.com.br/1Vvc0kOdBn</v>
+      </c>
+      <c r="D25" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E25" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Loja Ebenezer</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Loja em Destaque - Até 60%</v>
+      </c>
+      <c r="C26" t="str">
+        <v>https://s.shopee.com.br/10zLPpQXCi</v>
+      </c>
+      <c r="D26" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E26" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>BAOJUN ELETRONICOS</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Loja em Destaque - Até 57%</v>
+      </c>
+      <c r="C27" t="str">
+        <v>https://s.shopee.com.br/1BIlc8Ptrl</v>
+      </c>
+      <c r="D27" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E27" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>DYUSAR Cosméticos</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Loja em Destaque - Até 56%</v>
+      </c>
+      <c r="C28" t="str">
+        <v>https://s.shopee.com.br/gMV1DRnsg</v>
+      </c>
+      <c r="D28" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E28" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Lulia Mimos e Presentes</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Loja em Destaque - Até 53,01%</v>
+      </c>
+      <c r="C29" t="str">
+        <v>https://s.shopee.com.br/qfvDWRAXj</v>
+      </c>
+      <c r="D29" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E29" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>GR STORE OFICIAL</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Loja em Destaque - Até 53%</v>
+      </c>
+      <c r="C30" t="str">
+        <v>https://s.shopee.com.br/LjecbT4Ye</v>
+      </c>
+      <c r="D30" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E30" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>NWA Suplementos</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Loja em Destaque - Até 54%</v>
+      </c>
+      <c r="C31" t="str">
+        <v>https://s.shopee.com.br/W34ouSRDh</v>
+      </c>
+      <c r="D31" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E31" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>VASSOURAS MANERBA</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Loja em Destaque - Até 53%</v>
+      </c>
+      <c r="C32" t="str">
+        <v>https://s.shopee.com.br/16oDzULEc</v>
+      </c>
+      <c r="D32" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E32" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>A&amp;R Produtos</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Loja em Destaque - Até 53%</v>
+      </c>
+      <c r="C33" t="str">
+        <v>https://s.shopee.com.br/BQEQIThtf</v>
+      </c>
+      <c r="D33" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E33" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Gfmotopecas</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Loja em Destaque - Até 53%</v>
+      </c>
+      <c r="C34" t="str">
+        <v>https://s.shopee.com.br/AKX0Wyr0Ge</v>
+      </c>
+      <c r="D34" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E34" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Ozion Concept</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Loja em Destaque - Até 53%</v>
+      </c>
+      <c r="C35" t="str">
+        <v>https://s.shopee.com.br/AUqQjHqMvh</v>
+      </c>
+      <c r="D35" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E35" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Stella Wear</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Loja em Destaque - Até 51%</v>
+      </c>
+      <c r="C36" t="str">
+        <v>https://s.shopee.com.br/9zuA8MsGwc</v>
+      </c>
+      <c r="D36" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E36" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>ELLE HOME &amp; TECH</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Loja em Destaque - Até 44%</v>
+      </c>
+      <c r="C37" t="str">
+        <v>https://s.shopee.com.br/AADaKfrdbf</v>
+      </c>
+      <c r="D37" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E37" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Caminho da Tendência 2023</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Loja em Destaque - Até 45%</v>
+      </c>
+      <c r="C38" t="str">
+        <v>https://s.shopee.com.br/9fHJjktXca</v>
+      </c>
+      <c r="D38" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E38" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>KIMIMO Calçados</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Loja em Destaque - Até 43%</v>
+      </c>
+      <c r="C39" t="str">
+        <v>https://s.shopee.com.br/9pajw3suHd</v>
+      </c>
+      <c r="D39" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E39" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>LUÍS CALÇADOS</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Loja em Destaque - Até 43%</v>
+      </c>
+      <c r="C40" t="str">
+        <v>https://s.shopee.com.br/9KeTL8uoIY</v>
+      </c>
+      <c r="D40" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E40" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>rkmultidecor</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Loja em Destaque - Até 43%</v>
+      </c>
+      <c r="C41" t="str">
+        <v>https://s.shopee.com.br/9UxtXRuAxb</v>
+      </c>
+      <c r="D41" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E41" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Chi-in - Varejo</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Loja em Destaque - Até 41%</v>
+      </c>
+      <c r="C42" t="str">
+        <v>https://s.shopee.com.br/901cwWw4yW</v>
+      </c>
+      <c r="D42" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E42" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>ARAMARCO COMERCIO E DISTRIBUIÇÃO</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Loja em Destaque - Até 41%</v>
+      </c>
+      <c r="C43" t="str">
+        <v>https://s.shopee.com.br/9AL38pvRdZ</v>
+      </c>
+      <c r="D43" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E43" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>DÚ CAPAS ACESSÓRIOS AUTOMOTIVOS</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Loja em Destaque - Até 42%</v>
+      </c>
+      <c r="C44" t="str">
+        <v>https://s.shopee.com.br/8fOmXuxLeU</v>
+      </c>
+      <c r="D44" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E44" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>SLOTH SPORTING</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Loja em Destaque - Até 40%</v>
+      </c>
+      <c r="C45" t="str">
+        <v>https://s.shopee.com.br/8piCkDwiJX</v>
+      </c>
+      <c r="D45" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E45" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>De Paula Decor</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Loja em Destaque - Até 40%</v>
+      </c>
+      <c r="C46" t="str">
+        <v>https://s.shopee.com.br/8Klw9IycKS</v>
+      </c>
+      <c r="D46" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E46" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Farma super popular vilanova</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Loja em Destaque - Até 41%</v>
+      </c>
+      <c r="C47" t="str">
+        <v>https://s.shopee.com.br/8V5MLbxyzV</v>
+      </c>
+      <c r="D47" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E47" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>ESSENZIALE FARMA</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Loja em Destaque - Até 38%</v>
+      </c>
+      <c r="C48" t="str">
+        <v>https://s.shopee.com.br/8095kgzt0Q</v>
+      </c>
+      <c r="D48" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E48" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>J&amp;BP Imports</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Loja em Destaque - Até 38%</v>
+      </c>
+      <c r="C49" t="str">
+        <v>https://s.shopee.com.br/8ASVwzzFfT</v>
+      </c>
+      <c r="D49" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E49" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>FNW Distribuidora</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Loja em Destaque - Até 38%</v>
+      </c>
+      <c r="C50" t="str">
+        <v>https://s.shopee.com.br/7fWFM519gO</v>
+      </c>
+      <c r="D50" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E50" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Top Loja</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>JLF Utilidades Do Lar</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Loja em Destaque - Até 38%</v>
+      </c>
+      <c r="C51" t="str">
+        <v>https://s.shopee.com.br/7ppfYO0WLR</v>
+      </c>
+      <c r="D51" t="str">
+        <v>shopping-bag</v>
+      </c>
+      <c r="E51" t="str">
+        <v>#f53d2d</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Top Loja</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reformulacao visual Premium e atualizacao de produtos Shopee
</commit_message>
<xml_diff>
--- a/shopee.xlsx
+++ b/shopee.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Links" sheetId="1" r:id="rId1"/>
+    <sheet name="Produtos" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:F51"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,19 +410,13 @@
         <v>Link</v>
       </c>
       <c r="D1" t="str">
-        <v>Icone</v>
+        <v>Preco</v>
       </c>
       <c r="E1" t="str">
-        <v>CorIcone</v>
+        <v>Imagem</v>
       </c>
       <c r="F1" t="str">
         <v>Badge</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Imagem</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Preco</v>
       </c>
     </row>
     <row r="2">
@@ -430,25 +424,19 @@
         <v>LAA COSMÉTICOS</v>
       </c>
       <c r="B2" t="str">
-        <v>Loja em Destaque - Até 83%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
       </c>
       <c r="C2" t="str">
         <v>https://s.shopee.com.br/50VUBBBJ56</v>
       </c>
       <c r="D2" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E2" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F2" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G2" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="3">
@@ -456,25 +444,19 @@
         <v>The Foods</v>
       </c>
       <c r="B3" t="str">
-        <v>Loja em Destaque - Até 83%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
       </c>
       <c r="C3" t="str">
         <v>https://s.shopee.com.br/5AouNUAfk9</v>
       </c>
       <c r="D3" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E3" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F3" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G3" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="4">
@@ -482,25 +464,19 @@
         <v>Helô Naturais</v>
       </c>
       <c r="B4" t="str">
-        <v>Loja em Destaque - Até 83%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
       </c>
       <c r="C4" t="str">
         <v>https://s.shopee.com.br/4fsdmZCZl4</v>
       </c>
       <c r="D4" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E4" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F4" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G4" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="5">
@@ -508,25 +484,19 @@
         <v>Alfa Colors</v>
       </c>
       <c r="B5" t="str">
-        <v>Loja em Destaque - Até 83%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
       </c>
       <c r="C5" t="str">
         <v>https://s.shopee.com.br/4qC3ysBwQ7</v>
       </c>
       <c r="D5" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E5" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F5" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G5" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="6">
@@ -534,25 +504,19 @@
         <v>isabella vendas</v>
       </c>
       <c r="B6" t="str">
-        <v>Loja em Destaque - Até 83%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
       </c>
       <c r="C6" t="str">
         <v>https://s.shopee.com.br/4LFnNxDqR2</v>
       </c>
       <c r="D6" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E6" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F6" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G6" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="7">
@@ -560,25 +524,19 @@
         <v>MALUKA MODAS</v>
       </c>
       <c r="B7" t="str">
-        <v>Loja em Destaque - Até 83%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
       </c>
       <c r="C7" t="str">
         <v>https://s.shopee.com.br/4VZDaGDD65</v>
       </c>
       <c r="D7" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E7" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F7" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G7" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="8">
@@ -586,25 +544,19 @@
         <v>Fruttato</v>
       </c>
       <c r="B8" t="str">
-        <v>Loja em Destaque - Até 83%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
       </c>
       <c r="C8" t="str">
         <v>https://s.shopee.com.br/40cwzLF770</v>
       </c>
       <c r="D8" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E8" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F8" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G8" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="9">
@@ -612,25 +564,19 @@
         <v>detecidos</v>
       </c>
       <c r="B9" t="str">
-        <v>Loja em Destaque - Até 83%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
       </c>
       <c r="C9" t="str">
         <v>https://s.shopee.com.br/4AwNBeETm3</v>
       </c>
       <c r="D9" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E9" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F9" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G9" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H9" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="10">
@@ -638,25 +584,19 @@
         <v>Departamento Paulista Store</v>
       </c>
       <c r="B10" t="str">
-        <v>Loja em Destaque - Até 83%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
       </c>
       <c r="C10" t="str">
         <v>https://s.shopee.com.br/3g06ajGNmy</v>
       </c>
       <c r="D10" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E10" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F10" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G10" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H10" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="11">
@@ -664,25 +604,19 @@
         <v>Shop Fácil Store</v>
       </c>
       <c r="B11" t="str">
-        <v>Loja em Destaque - Até 82%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 82%)</v>
       </c>
       <c r="C11" t="str">
         <v>https://s.shopee.com.br/3qJWn2FkS1</v>
       </c>
       <c r="D11" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E11" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F11" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G11" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H11" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="12">
@@ -690,25 +624,19 @@
         <v>Mato Grosso Naturais</v>
       </c>
       <c r="B12" t="str">
-        <v>Loja em Destaque - Até 82%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 82%)</v>
       </c>
       <c r="C12" t="str">
         <v>https://s.shopee.com.br/3LNGC7HeSw</v>
       </c>
       <c r="D12" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E12" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F12" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G12" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H12" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="13">
@@ -716,25 +644,19 @@
         <v>Apolo Decor</v>
       </c>
       <c r="B13" t="str">
-        <v>Loja em Destaque - Até 80%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 80%)</v>
       </c>
       <c r="C13" t="str">
         <v>https://s.shopee.com.br/3VggOQH17z</v>
       </c>
       <c r="D13" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E13" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F13" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G13" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H13" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="14">
@@ -742,25 +664,19 @@
         <v>* TopVendarj *</v>
       </c>
       <c r="B14" t="str">
-        <v>Loja em Destaque - Até 80%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 80%)</v>
       </c>
       <c r="C14" t="str">
         <v>https://s.shopee.com.br/30kPnVIv8u</v>
       </c>
       <c r="D14" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E14" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F14" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G14" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H14" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="15">
@@ -768,25 +684,19 @@
         <v>Comercial SD Eletro-Eletrônico</v>
       </c>
       <c r="B15" t="str">
-        <v>Loja em Destaque - Até 78%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 78%)</v>
       </c>
       <c r="C15" t="str">
         <v>https://s.shopee.com.br/3B3pzoIHnx</v>
       </c>
       <c r="D15" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E15" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F15" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G15" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H15" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="16">
@@ -794,25 +704,19 @@
         <v>FÊNIX FRF</v>
       </c>
       <c r="B16" t="str">
-        <v>Loja em Destaque - Até 77%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 77%)</v>
       </c>
       <c r="C16" t="str">
         <v>https://s.shopee.com.br/2g7ZOtKBos</v>
       </c>
       <c r="D16" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E16" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F16" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G16" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H16" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="17">
@@ -820,25 +724,19 @@
         <v>TTL PAINEIS E ARTESANATO</v>
       </c>
       <c r="B17" t="str">
-        <v>Loja em Destaque - Até 73%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 73%)</v>
       </c>
       <c r="C17" t="str">
         <v>https://s.shopee.com.br/2qQzbCJYTv</v>
       </c>
       <c r="D17" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E17" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F17" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G17" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H17" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="18">
@@ -846,25 +744,19 @@
         <v>Viking Repelentes</v>
       </c>
       <c r="B18" t="str">
-        <v>Loja em Destaque - Até 73%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 73%)</v>
       </c>
       <c r="C18" t="str">
         <v>https://s.shopee.com.br/2LUj0HLSUq</v>
       </c>
       <c r="D18" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E18" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F18" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G18" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H18" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="19">
@@ -872,25 +764,19 @@
         <v>Márcia Cardoso de Oliveira lima</v>
       </c>
       <c r="B19" t="str">
-        <v>Loja em Destaque - Até 71%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 71%)</v>
       </c>
       <c r="C19" t="str">
         <v>https://s.shopee.com.br/2Vo9CaKp9t</v>
       </c>
       <c r="D19" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E19" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F19" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G19" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H19" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="20">
@@ -898,25 +784,19 @@
         <v>Tomate Racing33</v>
       </c>
       <c r="B20" t="str">
-        <v>Loja em Destaque - Até 69%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 69%)</v>
       </c>
       <c r="C20" t="str">
         <v>https://s.shopee.com.br/20rsbfMjAo</v>
       </c>
       <c r="D20" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E20" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F20" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G20" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H20" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="21">
@@ -924,25 +804,19 @@
         <v>Fernandes_Arts</v>
       </c>
       <c r="B21" t="str">
-        <v>Loja em Destaque - Até 68,78%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 68,78%)</v>
       </c>
       <c r="C21" t="str">
         <v>https://s.shopee.com.br/2BBInyM5pr</v>
       </c>
       <c r="D21" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E21" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F21" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G21" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H21" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="22">
@@ -950,25 +824,19 @@
         <v>Galera Adesivos</v>
       </c>
       <c r="B22" t="str">
-        <v>Loja em Destaque - Até 66,78%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 66,78%)</v>
       </c>
       <c r="C22" t="str">
         <v>https://s.shopee.com.br/1gF2D3Nzqm</v>
       </c>
       <c r="D22" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E22" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F22" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G22" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H22" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="23">
@@ -976,25 +844,19 @@
         <v>We Curve Estilos</v>
       </c>
       <c r="B23" t="str">
-        <v>Loja em Destaque - Até 63%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 63%)</v>
       </c>
       <c r="C23" t="str">
         <v>https://s.shopee.com.br/1qYSPMNMVp</v>
       </c>
       <c r="D23" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E23" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F23" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G23" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H23" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="24">
@@ -1002,25 +864,19 @@
         <v>STD Nutraceuticals</v>
       </c>
       <c r="B24" t="str">
-        <v>Loja em Destaque - Até 62%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 62%)</v>
       </c>
       <c r="C24" t="str">
         <v>https://s.shopee.com.br/1LcBoRPGWk</v>
       </c>
       <c r="D24" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E24" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F24" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G24" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H24" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="25">
@@ -1028,25 +884,19 @@
         <v>To Aqui Shop</v>
       </c>
       <c r="B25" t="str">
-        <v>Loja em Destaque - Até 62%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 62%)</v>
       </c>
       <c r="C25" t="str">
         <v>https://s.shopee.com.br/1Vvc0kOdBn</v>
       </c>
       <c r="D25" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E25" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F25" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G25" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H25" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="26">
@@ -1054,25 +904,19 @@
         <v>Loja Ebenezer</v>
       </c>
       <c r="B26" t="str">
-        <v>Loja em Destaque - Até 60%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 60%)</v>
       </c>
       <c r="C26" t="str">
         <v>https://s.shopee.com.br/10zLPpQXCi</v>
       </c>
       <c r="D26" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E26" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F26" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G26" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H26" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="27">
@@ -1080,25 +924,19 @@
         <v>BAOJUN ELETRONICOS</v>
       </c>
       <c r="B27" t="str">
-        <v>Loja em Destaque - Até 57%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 57%)</v>
       </c>
       <c r="C27" t="str">
         <v>https://s.shopee.com.br/1BIlc8Ptrl</v>
       </c>
       <c r="D27" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E27" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F27" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G27" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H27" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="28">
@@ -1106,25 +944,19 @@
         <v>DYUSAR Cosméticos</v>
       </c>
       <c r="B28" t="str">
-        <v>Loja em Destaque - Até 56%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 56%)</v>
       </c>
       <c r="C28" t="str">
         <v>https://s.shopee.com.br/gMV1DRnsg</v>
       </c>
       <c r="D28" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E28" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F28" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G28" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H28" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="29">
@@ -1132,25 +964,19 @@
         <v>Lulia Mimos e Presentes</v>
       </c>
       <c r="B29" t="str">
-        <v>Loja em Destaque - Até 53,01%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 53,01%)</v>
       </c>
       <c r="C29" t="str">
         <v>https://s.shopee.com.br/qfvDWRAXj</v>
       </c>
       <c r="D29" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E29" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F29" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G29" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H29" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="30">
@@ -1158,25 +984,19 @@
         <v>GR STORE OFICIAL</v>
       </c>
       <c r="B30" t="str">
-        <v>Loja em Destaque - Até 53%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 53%)</v>
       </c>
       <c r="C30" t="str">
         <v>https://s.shopee.com.br/LjecbT4Ye</v>
       </c>
       <c r="D30" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E30" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F30" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G30" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H30" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="31">
@@ -1184,25 +1004,19 @@
         <v>NWA Suplementos</v>
       </c>
       <c r="B31" t="str">
-        <v>Loja em Destaque - Até 54%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 54%)</v>
       </c>
       <c r="C31" t="str">
         <v>https://s.shopee.com.br/W34ouSRDh</v>
       </c>
       <c r="D31" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E31" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F31" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G31" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H31" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="32">
@@ -1210,25 +1024,19 @@
         <v>VASSOURAS MANERBA</v>
       </c>
       <c r="B32" t="str">
-        <v>Loja em Destaque - Até 53%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 53%)</v>
       </c>
       <c r="C32" t="str">
         <v>https://s.shopee.com.br/16oDzULEc</v>
       </c>
       <c r="D32" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E32" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F32" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G32" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H32" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="33">
@@ -1236,25 +1044,19 @@
         <v>A&amp;R Produtos</v>
       </c>
       <c r="B33" t="str">
-        <v>Loja em Destaque - Até 53%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 53%)</v>
       </c>
       <c r="C33" t="str">
         <v>https://s.shopee.com.br/BQEQIThtf</v>
       </c>
       <c r="D33" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E33" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F33" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G33" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H33" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="34">
@@ -1262,25 +1064,19 @@
         <v>Gfmotopecas</v>
       </c>
       <c r="B34" t="str">
-        <v>Loja em Destaque - Até 53%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 53%)</v>
       </c>
       <c r="C34" t="str">
         <v>https://s.shopee.com.br/AKX0Wyr0Ge</v>
       </c>
       <c r="D34" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E34" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F34" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G34" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H34" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="35">
@@ -1288,25 +1084,19 @@
         <v>Ozion Concept</v>
       </c>
       <c r="B35" t="str">
-        <v>Loja em Destaque - Até 53%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 53%)</v>
       </c>
       <c r="C35" t="str">
         <v>https://s.shopee.com.br/AUqQjHqMvh</v>
       </c>
       <c r="D35" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E35" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F35" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G35" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H35" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="36">
@@ -1314,25 +1104,19 @@
         <v>Stella Wear</v>
       </c>
       <c r="B36" t="str">
-        <v>Loja em Destaque - Até 51%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 51%)</v>
       </c>
       <c r="C36" t="str">
         <v>https://s.shopee.com.br/9zuA8MsGwc</v>
       </c>
       <c r="D36" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E36" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F36" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G36" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H36" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="37">
@@ -1340,25 +1124,19 @@
         <v>ELLE HOME &amp; TECH</v>
       </c>
       <c r="B37" t="str">
-        <v>Loja em Destaque - Até 44%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 44%)</v>
       </c>
       <c r="C37" t="str">
         <v>https://s.shopee.com.br/AADaKfrdbf</v>
       </c>
       <c r="D37" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E37" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F37" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G37" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H37" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="38">
@@ -1366,25 +1144,19 @@
         <v>Caminho da Tendência 2023</v>
       </c>
       <c r="B38" t="str">
-        <v>Loja em Destaque - Até 45%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 45%)</v>
       </c>
       <c r="C38" t="str">
         <v>https://s.shopee.com.br/9fHJjktXca</v>
       </c>
       <c r="D38" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E38" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F38" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G38" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H38" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="39">
@@ -1392,25 +1164,19 @@
         <v>KIMIMO Calçados</v>
       </c>
       <c r="B39" t="str">
-        <v>Loja em Destaque - Até 43%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 43%)</v>
       </c>
       <c r="C39" t="str">
         <v>https://s.shopee.com.br/9pajw3suHd</v>
       </c>
       <c r="D39" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E39" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F39" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G39" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H39" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="40">
@@ -1418,25 +1184,19 @@
         <v>LUÍS CALÇADOS</v>
       </c>
       <c r="B40" t="str">
-        <v>Loja em Destaque - Até 43%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 43%)</v>
       </c>
       <c r="C40" t="str">
         <v>https://s.shopee.com.br/9KeTL8uoIY</v>
       </c>
       <c r="D40" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E40" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F40" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G40" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H40" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="41">
@@ -1444,25 +1204,19 @@
         <v>rkmultidecor</v>
       </c>
       <c r="B41" t="str">
-        <v>Loja em Destaque - Até 43%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 43%)</v>
       </c>
       <c r="C41" t="str">
         <v>https://s.shopee.com.br/9UxtXRuAxb</v>
       </c>
       <c r="D41" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E41" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F41" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G41" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H41" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="42">
@@ -1470,25 +1224,19 @@
         <v>Chi-in - Varejo</v>
       </c>
       <c r="B42" t="str">
-        <v>Loja em Destaque - Até 41%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 41%)</v>
       </c>
       <c r="C42" t="str">
         <v>https://s.shopee.com.br/901cwWw4yW</v>
       </c>
       <c r="D42" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E42" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F42" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G42" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H42" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="43">
@@ -1496,25 +1244,19 @@
         <v>ARAMARCO COMERCIO E DISTRIBUIÇÃO</v>
       </c>
       <c r="B43" t="str">
-        <v>Loja em Destaque - Até 41%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 41%)</v>
       </c>
       <c r="C43" t="str">
         <v>https://s.shopee.com.br/9AL38pvRdZ</v>
       </c>
       <c r="D43" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E43" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F43" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G43" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H43" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="44">
@@ -1522,25 +1264,19 @@
         <v>DÚ CAPAS ACESSÓRIOS AUTOMOTIVOS</v>
       </c>
       <c r="B44" t="str">
-        <v>Loja em Destaque - Até 42%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 42%)</v>
       </c>
       <c r="C44" t="str">
         <v>https://s.shopee.com.br/8fOmXuxLeU</v>
       </c>
       <c r="D44" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E44" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F44" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G44" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H44" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="45">
@@ -1548,25 +1284,19 @@
         <v>SLOTH SPORTING</v>
       </c>
       <c r="B45" t="str">
-        <v>Loja em Destaque - Até 40%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 40%)</v>
       </c>
       <c r="C45" t="str">
         <v>https://s.shopee.com.br/8piCkDwiJX</v>
       </c>
       <c r="D45" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E45" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F45" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G45" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H45" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="46">
@@ -1574,25 +1304,19 @@
         <v>De Paula Decor</v>
       </c>
       <c r="B46" t="str">
-        <v>Loja em Destaque - Até 40%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 40%)</v>
       </c>
       <c r="C46" t="str">
         <v>https://s.shopee.com.br/8Klw9IycKS</v>
       </c>
       <c r="D46" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E46" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F46" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G46" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H46" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="47">
@@ -1600,25 +1324,19 @@
         <v>Farma super popular vilanova</v>
       </c>
       <c r="B47" t="str">
-        <v>Loja em Destaque - Até 41%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 41%)</v>
       </c>
       <c r="C47" t="str">
         <v>https://s.shopee.com.br/8V5MLbxyzV</v>
       </c>
       <c r="D47" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E47" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F47" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G47" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H47" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="48">
@@ -1626,25 +1344,19 @@
         <v>ESSENZIALE FARMA</v>
       </c>
       <c r="B48" t="str">
-        <v>Loja em Destaque - Até 38%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 38%)</v>
       </c>
       <c r="C48" t="str">
         <v>https://s.shopee.com.br/8095kgzt0Q</v>
       </c>
       <c r="D48" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E48" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F48" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G48" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H48" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="49">
@@ -1652,25 +1364,19 @@
         <v>J&amp;BP Imports</v>
       </c>
       <c r="B49" t="str">
-        <v>Loja em Destaque - Até 38%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 38%)</v>
       </c>
       <c r="C49" t="str">
         <v>https://s.shopee.com.br/8ASVwzzFfT</v>
       </c>
       <c r="D49" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E49" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F49" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G49" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H49" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="50">
@@ -1678,25 +1384,19 @@
         <v>FNW Distribuidora</v>
       </c>
       <c r="B50" t="str">
-        <v>Loja em Destaque - Até 38%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 38%)</v>
       </c>
       <c r="C50" t="str">
         <v>https://s.shopee.com.br/7fWFM519gO</v>
       </c>
       <c r="D50" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E50" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F50" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G50" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H50" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
     <row r="51">
@@ -1704,30 +1404,24 @@
         <v>JLF Utilidades Do Lar</v>
       </c>
       <c r="B51" t="str">
-        <v>Loja em Destaque - Até 38%</v>
+        <v>Oferta Especial Shopee (Comissão: up to 38%)</v>
       </c>
       <c r="C51" t="str">
         <v>https://s.shopee.com.br/7ppfYO0WLR</v>
       </c>
       <c r="D51" t="str">
-        <v>shopping-bag</v>
+        <v>R$ Ver Preço</v>
       </c>
       <c r="E51" t="str">
-        <v>#f53d2d</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F51" t="str">
-        <v>Top Loja</v>
-      </c>
-      <c r="G51" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
-      </c>
-      <c r="H51" t="str">
-        <v>Ver Loja</v>
+        <v>Shopee</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Importação de 100 novos produtos individuais da Shopee
</commit_message>
<xml_diff>
--- a/shopee.xlsx
+++ b/shopee.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F101"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,16 +421,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>LAA COSMÉTICOS</v>
+        <v>40 Peças / 46 Peças Jogo De Chave Catraca Caixa De Ferramentas Completa Reversível Soquetes Maleta</v>
       </c>
       <c r="B2" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.19)</v>
       </c>
       <c r="C2" t="str">
-        <v>https://s.shopee.com.br/50VUBBBJ56</v>
+        <v>https://s.shopee.com.br/2BBKKZxaPL</v>
       </c>
       <c r="D2" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 3099</v>
       </c>
       <c r="E2" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -441,16 +441,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>The Foods</v>
+        <v>Kit  Collagen Completo Máscara 500g Shampoo 1L Condicionador 1L Óleo Maca 50ml Tratamento Profissional</v>
       </c>
       <c r="B3" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.16)</v>
       </c>
       <c r="C3" t="str">
-        <v>https://s.shopee.com.br/5AouNUAfk9</v>
+        <v>https://s.shopee.com.br/1gF3jezUQG</v>
       </c>
       <c r="D3" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 5400</v>
       </c>
       <c r="E3" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -461,16 +461,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Helô Naturais</v>
+        <v>Jogo de Lençol 400 Fios Cama Solteiro Casal Queen King E Berço Micropercal Ponto Palito</v>
       </c>
       <c r="B4" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.21)</v>
       </c>
       <c r="C4" t="str">
-        <v>https://s.shopee.com.br/4fsdmZCZl4</v>
+        <v>https://s.shopee.com.br/1qYTvxyr5J</v>
       </c>
       <c r="D4" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 2723</v>
       </c>
       <c r="E4" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -481,16 +481,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Alfa Colors</v>
+        <v>Kit 1 ou 2 Unidades de Veda Porta Ajustável Protetor Rolinho Impermeável 80cm 90cm 100cm</v>
       </c>
       <c r="B5" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.24)</v>
       </c>
       <c r="C5" t="str">
-        <v>https://s.shopee.com.br/4qC3ysBwQ7</v>
+        <v>https://s.shopee.com.br/1LcDL30l6E</v>
       </c>
       <c r="D5" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1254</v>
       </c>
       <c r="E5" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -501,16 +501,16 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>isabella vendas</v>
+        <v>Kit Limpador Pastilha de máquina de lavar roupa, comprimido efervescente sólido para remover manchas【】</v>
       </c>
       <c r="B6" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
       </c>
       <c r="C6" t="str">
-        <v>https://s.shopee.com.br/4LFnNxDqR2</v>
+        <v>https://s.shopee.com.br/1VvdXM07lH</v>
       </c>
       <c r="D6" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 859</v>
       </c>
       <c r="E6" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -521,16 +521,16 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MALUKA MODAS</v>
+        <v>Kit 3 Peneira Coador De Peneiras Aço Inoxidável Para Cozinha Peneira De Cozinha</v>
       </c>
       <c r="B7" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.15)</v>
       </c>
       <c r="C7" t="str">
-        <v>https://s.shopee.com.br/4VZDaGDD65</v>
+        <v>https://s.shopee.com.br/3g087KrsMi</v>
       </c>
       <c r="D7" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1599</v>
       </c>
       <c r="E7" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -541,16 +541,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Fruttato</v>
+        <v>Inox Torneira  Prata/Preto Com Chuveiro Com Rotação De 360° Cozinha Luxo Parede Promoção</v>
       </c>
       <c r="B8" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
       </c>
       <c r="C8" t="str">
-        <v>https://s.shopee.com.br/40cwzLF770</v>
+        <v>https://s.shopee.com.br/3qJYJdrF1l</v>
       </c>
       <c r="D8" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 2399</v>
       </c>
       <c r="E8" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -561,16 +561,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>detecidos</v>
+        <v>KIT 1/2/5 Suporte De Parede Multifuncional Caixa De Armazenamento Casa Para Carregar Remoto Um Slot Promoção</v>
       </c>
       <c r="B9" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
       </c>
       <c r="C9" t="str">
-        <v>https://s.shopee.com.br/4AwNBeETm3</v>
+        <v>https://s.shopee.com.br/3LNHiit92g</v>
       </c>
       <c r="D9" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 959</v>
       </c>
       <c r="E9" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -581,16 +581,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Departamento Paulista Store</v>
+        <v>Mangueira de Jardim Anti-Torção e Anti-Dobras de 5 a 50 Metros</v>
       </c>
       <c r="B10" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 83%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.21)</v>
       </c>
       <c r="C10" t="str">
-        <v>https://s.shopee.com.br/3g06ajGNmy</v>
+        <v>https://s.shopee.com.br/3Vghv1sVhj</v>
       </c>
       <c r="D10" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1732</v>
       </c>
       <c r="E10" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -601,16 +601,16 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Shop Fácil Store</v>
+        <v>Creme Desodorante Antitranspirante Herbíssimo Care Rosa Mosqueta E Niacinamida Bisnaga 55g</v>
       </c>
       <c r="B11" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 82%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.17)</v>
       </c>
       <c r="C11" t="str">
-        <v>https://s.shopee.com.br/3qJWn2FkS1</v>
+        <v>https://s.shopee.com.br/30kRK6uPie</v>
       </c>
       <c r="D11" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1699</v>
       </c>
       <c r="E11" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -621,16 +621,16 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Mato Grosso Naturais</v>
+        <v>Kit Maca Power Completo com 7 Produtos – Cronograma Capilar + Máscara 500g, Shampoo 1L, Condicionador 1L  Reparador 50ml</v>
       </c>
       <c r="B12" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 82%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.16)</v>
       </c>
       <c r="C12" t="str">
-        <v>https://s.shopee.com.br/3LNGC7HeSw</v>
+        <v>https://s.shopee.com.br/3B3rWPtmNh</v>
       </c>
       <c r="D12" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 7800</v>
       </c>
       <c r="E12" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -641,16 +641,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Apolo Decor</v>
+        <v>Creme Depilatório Corporal Depilsam Aloe Vera 200G</v>
       </c>
       <c r="B13" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 80%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.17)</v>
       </c>
       <c r="C13" t="str">
-        <v>https://s.shopee.com.br/3VggOQH17z</v>
+        <v>https://s.shopee.com.br/2g7avUvgOc</v>
       </c>
       <c r="D13" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 2498</v>
       </c>
       <c r="E13" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -661,16 +661,16 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>* TopVendarj *</v>
+        <v>Protetor de Colchão Impermeável Matelado Varias Cores Para Cama Box Solteiro, Casal, Queen, King, Mini Berço E Berço</v>
       </c>
       <c r="B14" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 80%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.24)</v>
       </c>
       <c r="C14" t="str">
-        <v>https://s.shopee.com.br/30kPnVIv8u</v>
+        <v>https://s.shopee.com.br/2qR17nv33f</v>
       </c>
       <c r="D14" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1590</v>
       </c>
       <c r="E14" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -681,16 +681,16 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Comercial SD Eletro-Eletrônico</v>
+        <v>KIT 3, 6 e 9 Calcinha Feminina Tanga Infantil Juvenil Algodão Macio Ajuste Perfeito Cores Estampas Sortidas</v>
       </c>
       <c r="B15" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 78%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
       </c>
       <c r="C15" t="str">
-        <v>https://s.shopee.com.br/3B3pzoIHnx</v>
+        <v>https://s.shopee.com.br/50VVhmmnf6</v>
       </c>
       <c r="D15" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1590</v>
       </c>
       <c r="E15" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -701,16 +701,16 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>FÊNIX FRF</v>
+        <v>JBSARA Soro Renovador de Retinol 1ml Envio da Coreia 1 peça</v>
       </c>
       <c r="B16" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 77%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.15)</v>
       </c>
       <c r="C16" t="str">
-        <v>https://s.shopee.com.br/2g7ZOtKBos</v>
+        <v>https://s.shopee.com.br/5Aovu5mAK9</v>
       </c>
       <c r="D16" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 349</v>
       </c>
       <c r="E16" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -721,16 +721,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>TTL PAINEIS E ARTESANATO</v>
+        <v>Regata Alça Fina Fitness Blusa Feminino Liso Poliamida Tank Top Slim Camiseta Academia Verão</v>
       </c>
       <c r="B17" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 73%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.19)</v>
       </c>
       <c r="C17" t="str">
-        <v>https://s.shopee.com.br/2qQzbCJYTv</v>
+        <v>https://s.shopee.com.br/4fsfJAo4L4</v>
       </c>
       <c r="D17" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 3790</v>
       </c>
       <c r="E17" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -741,16 +741,16 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Viking Repelentes</v>
+        <v>Fórmula de Lyah 60 doses - Suplemento Alimentar</v>
       </c>
       <c r="B18" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 73%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.25)</v>
       </c>
       <c r="C18" t="str">
-        <v>https://s.shopee.com.br/2LUj0HLSUq</v>
+        <v>https://s.shopee.com.br/4qC5VTnR07</v>
       </c>
       <c r="D18" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 6990</v>
       </c>
       <c r="E18" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -761,16 +761,16 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Márcia Cardoso de Oliveira lima</v>
+        <v>Creme Gel Regenerador Facial Gota de Colágeno Kokeshi 45g</v>
       </c>
       <c r="B19" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 71%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.24)</v>
       </c>
       <c r="C19" t="str">
-        <v>https://s.shopee.com.br/2Vo9CaKp9t</v>
+        <v>https://s.shopee.com.br/4LFouYpL12</v>
       </c>
       <c r="D19" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 3283</v>
       </c>
       <c r="E19" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -781,16 +781,16 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Tomate Racing33</v>
+        <v>Creme Para Pentear Definição Natural 1kg</v>
       </c>
       <c r="B20" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 69%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
       </c>
       <c r="C20" t="str">
-        <v>https://s.shopee.com.br/20rsbfMjAo</v>
+        <v>https://s.shopee.com.br/4VZF6rohg5</v>
       </c>
       <c r="D20" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 3575</v>
       </c>
       <c r="E20" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -801,16 +801,16 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Fernandes_Arts</v>
+        <v>Cinta Modeladora Espartilho De Emagrecimento-ENVIO IMEDIATO --8888</v>
       </c>
       <c r="B21" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 68,78%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.16)</v>
       </c>
       <c r="C21" t="str">
-        <v>https://s.shopee.com.br/2BBInyM5pr</v>
+        <v>https://s.shopee.com.br/40cyVwqbh0</v>
       </c>
       <c r="D21" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 2280</v>
       </c>
       <c r="E21" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -821,16 +821,16 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Galera Adesivos</v>
+        <v>1/2/3 Forro Antiderrapante Para Gaveta, Geladeira E Guarda Roupas- Transparente 0,6*3M Evita Deslizamento em Superfícies</v>
       </c>
       <c r="B22" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 66,78%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.19)</v>
       </c>
       <c r="C22" t="str">
-        <v>https://s.shopee.com.br/1gF2D3Nzqm</v>
+        <v>https://s.shopee.com.br/4AwOiFpyM3</v>
       </c>
       <c r="D22" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 2399</v>
       </c>
       <c r="E22" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -841,16 +841,16 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>We Curve Estilos</v>
+        <v>Kit 10 Marmita conjunto Potes 750ml com Travas Laterais BPA FREE - Alimentos organizadores de congelador</v>
       </c>
       <c r="B23" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 63%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
       </c>
       <c r="C23" t="str">
-        <v>https://s.shopee.com.br/1qYSPMNMVp</v>
+        <v>https://s.shopee.com.br/6L0tIEhixU</v>
       </c>
       <c r="D23" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 2190</v>
       </c>
       <c r="E23" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -861,16 +861,16 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>STD Nutraceuticals</v>
+        <v>Relógio Masculino digital wr | 100 % qualidade | entrega rápida</v>
       </c>
       <c r="B24" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 62%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
       </c>
       <c r="C24" t="str">
-        <v>https://s.shopee.com.br/1LcBoRPGWk</v>
+        <v>https://s.shopee.com.br/6VKJUXh5cX</v>
       </c>
       <c r="D24" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1299</v>
       </c>
       <c r="E24" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -881,16 +881,16 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>To Aqui Shop</v>
+        <v>Coberdrom Cobertor Solteiro Casal Queen E King Colcha Dupla Face Edredrom Luxo Pele Carneiro Premium</v>
       </c>
       <c r="B25" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 62%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
       </c>
       <c r="C25" t="str">
-        <v>https://s.shopee.com.br/1Vvc0kOdBn</v>
+        <v>https://s.shopee.com.br/60O2tcizdS</v>
       </c>
       <c r="D25" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 9498</v>
       </c>
       <c r="E25" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -901,16 +901,16 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Loja Ebenezer</v>
+        <v>Amplificador De Imagem Da Tela Do Celular Lupa 3D 21,6CM*16,6CM*2,7CM Promoção</v>
       </c>
       <c r="B26" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 60%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
       </c>
       <c r="C26" t="str">
-        <v>https://s.shopee.com.br/10zLPpQXCi</v>
+        <v>https://s.shopee.com.br/6AhT5viMIV</v>
       </c>
       <c r="D26" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1799</v>
       </c>
       <c r="E26" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -921,16 +921,16 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>BAOJUN ELETRONICOS</v>
+        <v>Óleo de Tratamento SOS Cachos 10 em 1 Multibenefícios 42ml</v>
       </c>
       <c r="B27" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 57%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
       </c>
       <c r="C27" t="str">
-        <v>https://s.shopee.com.br/1BIlc8Ptrl</v>
+        <v>https://s.shopee.com.br/5flCV0kGJQ</v>
       </c>
       <c r="D27" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1620</v>
       </c>
       <c r="E27" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -941,16 +941,16 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>DYUSAR Cosméticos</v>
+        <v>Arranjo c/ 3 Trepadeira Folha de HERA + Vaso Trançado Marrom</v>
       </c>
       <c r="B28" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 56%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.28)</v>
       </c>
       <c r="C28" t="str">
-        <v>https://s.shopee.com.br/gMV1DRnsg</v>
+        <v>https://s.shopee.com.br/5q4chJjcyT</v>
       </c>
       <c r="D28" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1680</v>
       </c>
       <c r="E28" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -961,16 +961,16 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Lulia Mimos e Presentes</v>
+        <v>Alvejante Poderoso com Percarbonato de Sódio Tira Manchas Roupas Brancas e Coloridas -GF Agro</v>
       </c>
       <c r="B29" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 53,01%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.22)</v>
       </c>
       <c r="C29" t="str">
-        <v>https://s.shopee.com.br/qfvDWRAXj</v>
+        <v>https://s.shopee.com.br/5L8M6OlWzO</v>
       </c>
       <c r="D29" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1199</v>
       </c>
       <c r="E29" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -981,16 +981,16 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>GR STORE OFICIAL</v>
+        <v>30 unidades cabide redondo resistente adulto</v>
       </c>
       <c r="B30" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 53%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.17)</v>
       </c>
       <c r="C30" t="str">
-        <v>https://s.shopee.com.br/LjecbT4Ye</v>
+        <v>https://s.shopee.com.br/5VRmIhkteR</v>
       </c>
       <c r="D30" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1998</v>
       </c>
       <c r="E30" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1001,16 +1001,16 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>NWA Suplementos</v>
+        <v>Principia Kit Completo Peles Sensíveis c/ Gel de Limpeza Gl-02 + Creme Hidratante CH-01 + Protetor Solar PS-01 FPS 60</v>
       </c>
       <c r="B31" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 54%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.15)</v>
       </c>
       <c r="C31" t="str">
-        <v>https://s.shopee.com.br/W34ouSRDh</v>
+        <v>https://s.shopee.com.br/7fWGsgceFs</v>
       </c>
       <c r="D31" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 11625</v>
       </c>
       <c r="E31" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1021,16 +1021,16 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>VASSOURAS MANERBA</v>
+        <v>Cera Espelhamento RENOVE – Remove Riscos Superficiais, Repele Água, Proteção Sol, Brilho Intenso</v>
       </c>
       <c r="B32" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 53%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.24)</v>
       </c>
       <c r="C32" t="str">
-        <v>https://s.shopee.com.br/16oDzULEc</v>
+        <v>https://s.shopee.com.br/7pph4zc0uv</v>
       </c>
       <c r="D32" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1799</v>
       </c>
       <c r="E32" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1041,16 +1041,16 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>A&amp;R Produtos</v>
+        <v>Kit 10, 5 Cueca Masculina Box Adulto Microfibra Forro 100% Algodão Cores Variadas</v>
       </c>
       <c r="B33" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 53%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
       </c>
       <c r="C33" t="str">
-        <v>https://s.shopee.com.br/BQEQIThtf</v>
+        <v>https://s.shopee.com.br/7KtQU4duvq</v>
       </c>
       <c r="D33" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 2680</v>
       </c>
       <c r="E33" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1061,16 +1061,16 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Gfmotopecas</v>
+        <v>Mini Umidificador Difusor Aromatizador Egg Portátil Usb Led Aromatizador De Ambiente Purificador De Ar Casa Escritório</v>
       </c>
       <c r="B34" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 53%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.19)</v>
       </c>
       <c r="C34" t="str">
-        <v>https://s.shopee.com.br/AKX0Wyr0Ge</v>
+        <v>https://s.shopee.com.br/7VCqgNdHat</v>
       </c>
       <c r="D34" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1699</v>
       </c>
       <c r="E34" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1081,16 +1081,16 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Ozion Concept</v>
+        <v>Luminária Despertador Com Luz Led Bluetooth Caixa  Som Relógio Digital  Carregamento Indução Abajur</v>
       </c>
       <c r="B35" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 53%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
       </c>
       <c r="C35" t="str">
-        <v>https://s.shopee.com.br/AUqQjHqMvh</v>
+        <v>https://s.shopee.com.br/70Ga5SfBbo</v>
       </c>
       <c r="D35" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 3490</v>
       </c>
       <c r="E35" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1101,16 +1101,16 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Stella Wear</v>
+        <v>kit Coala Home Chá Branco</v>
       </c>
       <c r="B36" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 51%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.19)</v>
       </c>
       <c r="C36" t="str">
-        <v>https://s.shopee.com.br/9zuA8MsGwc</v>
+        <v>https://s.shopee.com.br/7Aa0HleYGr</v>
       </c>
       <c r="D36" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 6999</v>
       </c>
       <c r="E36" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1121,16 +1121,16 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ELLE HOME &amp; TECH</v>
+        <v>Cafe Graos Torra Media Gourmet Café Italle 1kg</v>
       </c>
       <c r="B37" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 44%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.28)</v>
       </c>
       <c r="C37" t="str">
-        <v>https://s.shopee.com.br/AADaKfrdbf</v>
+        <v>https://s.shopee.com.br/6fdjgqgSHm</v>
       </c>
       <c r="D37" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 7130</v>
       </c>
       <c r="E37" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1141,16 +1141,16 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Caminho da Tendência 2023</v>
+        <v>Cinto Masculino Feminino Tecido Trançado Elástico Fivela De Metal</v>
       </c>
       <c r="B38" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 45%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.17)</v>
       </c>
       <c r="C38" t="str">
-        <v>https://s.shopee.com.br/9fHJjktXca</v>
+        <v>https://s.shopee.com.br/6px9t9fowp</v>
       </c>
       <c r="D38" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1099</v>
       </c>
       <c r="E38" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1161,16 +1161,16 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>KIMIMO Calçados</v>
+        <v>Kit de 72 unidades de Xuxinha de cabelo elastico de para cabelo feminino rabicó</v>
       </c>
       <c r="B39" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 43%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
       </c>
       <c r="C39" t="str">
-        <v>https://s.shopee.com.br/9pajw3suHd</v>
+        <v>https://s.shopee.com.br/901eT8XZYG</v>
       </c>
       <c r="D39" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1087</v>
       </c>
       <c r="E39" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1181,16 +1181,16 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>LUÍS CALÇADOS</v>
+        <v>Manta Cobertor Microfibra Casal Queen King Quentinha Antialérgico Poá Habitat</v>
       </c>
       <c r="B40" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 43%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.21)</v>
       </c>
       <c r="C40" t="str">
-        <v>https://s.shopee.com.br/9KeTL8uoIY</v>
+        <v>https://s.shopee.com.br/9AL4fRWwDJ</v>
       </c>
       <c r="D40" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 5289</v>
       </c>
       <c r="E40" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1201,16 +1201,16 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>rkmultidecor</v>
+        <v>Pistola Elétrica Para Pintura Pulverizador de Tinta com Bico de Metal e Compressor 450w - TSSAPER</v>
       </c>
       <c r="B41" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 43%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.15)</v>
       </c>
       <c r="C41" t="str">
-        <v>https://s.shopee.com.br/9UxtXRuAxb</v>
+        <v>https://s.shopee.com.br/8fOo4WYqEE</v>
       </c>
       <c r="D41" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 13745</v>
       </c>
       <c r="E41" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1221,16 +1221,16 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Chi-in - Varejo</v>
+        <v>Lençol Com Elástico Premium Avulso 400 Fios Percal Liso Toque Macio Acetinado</v>
       </c>
       <c r="B42" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 41%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
       </c>
       <c r="C42" t="str">
-        <v>https://s.shopee.com.br/901cwWw4yW</v>
+        <v>https://s.shopee.com.br/8piEGpYCtH</v>
       </c>
       <c r="D42" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1880</v>
       </c>
       <c r="E42" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1241,16 +1241,16 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ARAMARCO COMERCIO E DISTRIBUIÇÃO</v>
+        <v>Balança Corporal Transparente Quadrada Digital Até 180kg Com Vidro Temperado Premium</v>
       </c>
       <c r="B43" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 41%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.19)</v>
       </c>
       <c r="C43" t="str">
-        <v>https://s.shopee.com.br/9AL38pvRdZ</v>
+        <v>https://s.shopee.com.br/8Klxfua6uC</v>
       </c>
       <c r="D43" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 3299</v>
       </c>
       <c r="E43" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1261,16 +1261,16 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>DÚ CAPAS ACESSÓRIOS AUTOMOTIVOS</v>
+        <v>2025 Nova Série 8 Relógio T800 Ultra Smart Watch Esportivo Sem Fio À Prova D'água T800 Ultra2 MAX</v>
       </c>
       <c r="B44" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 42%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.16)</v>
       </c>
       <c r="C44" t="str">
-        <v>https://s.shopee.com.br/8fOmXuxLeU</v>
+        <v>https://s.shopee.com.br/8V5NsDZTZF</v>
       </c>
       <c r="D44" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 3899</v>
       </c>
       <c r="E44" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1281,16 +1281,16 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>SLOTH SPORTING</v>
+        <v>Protetor Solar Facial PS-01 FPS 60 Principia</v>
       </c>
       <c r="B45" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 40%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.15)</v>
       </c>
       <c r="C45" t="str">
-        <v>https://s.shopee.com.br/8piCkDwiJX</v>
+        <v>https://s.shopee.com.br/8097HIbNaA</v>
       </c>
       <c r="D45" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 4900</v>
       </c>
       <c r="E45" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1301,16 +1301,16 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>De Paula Decor</v>
+        <v>Leggings canelada de cintura larga e cor sólida para atividades esportivas.</v>
       </c>
       <c r="B46" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 40%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
       </c>
       <c r="C46" t="str">
-        <v>https://s.shopee.com.br/8Klw9IycKS</v>
+        <v>https://s.shopee.com.br/8ASXTbakFD</v>
       </c>
       <c r="D46" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 2999</v>
       </c>
       <c r="E46" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1321,16 +1321,16 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Farma super popular vilanova</v>
+        <v>Blusa Feminina Manga 3/4 Novas Cores Tecido Crepe Moda Evangelica Detalhe Social Elegante</v>
       </c>
       <c r="B47" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 41%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.34)</v>
       </c>
       <c r="C47" t="str">
-        <v>https://s.shopee.com.br/8V5MLbxyzV</v>
+        <v>https://s.shopee.com.br/AKX23aSUqe</v>
       </c>
       <c r="D47" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 2699</v>
       </c>
       <c r="E47" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1341,16 +1341,16 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ESSENZIALE FARMA</v>
+        <v>Fita Multiuso Manta Asfaltica Adesiva para Reparos Rufo Calha Telhado Veda Tudo 10cm 20cm 30cm POR METRO</v>
       </c>
       <c r="B48" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 38%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.16)</v>
       </c>
       <c r="C48" t="str">
-        <v>https://s.shopee.com.br/8095kgzt0Q</v>
+        <v>https://s.shopee.com.br/AUqSFtRrVh</v>
       </c>
       <c r="D48" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 999</v>
       </c>
       <c r="E48" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1361,16 +1361,16 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>J&amp;BP Imports</v>
+        <v>Blusa Manga 3/4 Detalhe Em V Novas Cores Verão Tendência Moda Feminina</v>
       </c>
       <c r="B49" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 38%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.17)</v>
       </c>
       <c r="C49" t="str">
-        <v>https://s.shopee.com.br/8ASVwzzFfT</v>
+        <v>https://s.shopee.com.br/9zuBeyTlWc</v>
       </c>
       <c r="D49" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 2699</v>
       </c>
       <c r="E49" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1381,16 +1381,16 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>FNW Distribuidora</v>
+        <v>Kit M10 Bluetooth 5.3 Sem Fio TWS Fones De Ouvido Estéreo Com Carregador Power Bank Atualizado 100 % Novo Alto-Falante</v>
       </c>
       <c r="B50" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 38%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.33)</v>
       </c>
       <c r="C50" t="str">
-        <v>https://s.shopee.com.br/7fWFM519gO</v>
+        <v>https://s.shopee.com.br/AADbrHT8Bf</v>
       </c>
       <c r="D50" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 2589</v>
       </c>
       <c r="E50" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
@@ -1401,27 +1401,1027 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>JLF Utilidades Do Lar</v>
+        <v>Shampoo Tonalizante Escurecedor S/ Amônia Avelã, Marsala, Loiro, Vermelho Ruivo 100% Natural Matizze</v>
       </c>
       <c r="B51" t="str">
-        <v>Oferta Especial Shopee (Comissão: up to 38%)</v>
+        <v>Oferta Especial Shopee (Comissão: 0.15)</v>
       </c>
       <c r="C51" t="str">
-        <v>https://s.shopee.com.br/7ppfYO0WLR</v>
+        <v>https://s.shopee.com.br/9fHLGMV2Ca</v>
       </c>
       <c r="D51" t="str">
-        <v>R$ Ver Preço</v>
+        <v>R$ 1789</v>
       </c>
       <c r="E51" t="str">
         <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
       </c>
       <c r="F51" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Kit de Óleo Capilar - Cronograma Terapia Capilar - 100% natural - 60ml</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.2)</v>
+      </c>
+      <c r="C52" t="str">
+        <v>https://s.shopee.com.br/9palSfUOrd</v>
+      </c>
+      <c r="D52" t="str">
+        <v>R$ 1530</v>
+      </c>
+      <c r="E52" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Carregador Portátil Mini Power Bank 10000mAh Com 02 Saídas Tipo-C / Lightning</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.34)</v>
+      </c>
+      <c r="C53" t="str">
+        <v>https://s.shopee.com.br/9KeUrkWIsY</v>
+      </c>
+      <c r="D53" t="str">
+        <v>R$ 3299</v>
+      </c>
+      <c r="E53" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Mini Barbeador Elétrico Portátil À Prova D'água De Dupla Finalidade Tipo c De Carga Rápida Aparador De Barba De Bolso</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
+      </c>
+      <c r="C54" t="str">
+        <v>https://s.shopee.com.br/9Uxv43VfXb</v>
+      </c>
+      <c r="D54" t="str">
+        <v>R$ 1699</v>
+      </c>
+      <c r="E54" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Trava Óculos Antiderrapante Silicone Kit Não Cai Do Rosto Gancho Orelha Haste Conforto</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C55" t="str">
+        <v>https://s.shopee.com.br/1BIn8k1OS0</v>
+      </c>
+      <c r="D55" t="str">
+        <v>R$ 700</v>
+      </c>
+      <c r="E55" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Kit 3 Bermudas Masculina Esportivo Academia Praia Com  Bolsos E Refletivo</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C56" t="str">
+        <v>https://s.shopee.com.br/10zMwR21mz</v>
+      </c>
+      <c r="D56" t="str">
+        <v>R$ 4404</v>
+      </c>
+      <c r="E56" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Kit Com 10 ou 4 Cuecas Boxers Premium Masculina Adulto de Microfibra</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.15)</v>
+      </c>
+      <c r="C57" t="str">
+        <v>https://s.shopee.com.br/qfwk82f7y</v>
+      </c>
+      <c r="D57" t="str">
+        <v>R$ 2498</v>
+      </c>
+      <c r="E57" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Shorts modeladores sem costura com forro de microfibra</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.16)</v>
+      </c>
+      <c r="C58" t="str">
+        <v>https://s.shopee.com.br/gMWXp3ISx</v>
+      </c>
+      <c r="D58" t="str">
+        <v>R$ 1924</v>
+      </c>
+      <c r="E58" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Kit 4pçs Toalhas de Banho 140x70cm 100% Algodão Premium Coleção Difiori</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.33)</v>
+      </c>
+      <c r="C59" t="str">
+        <v>https://s.shopee.com.br/W36LW3vnw</v>
+      </c>
+      <c r="D59" t="str">
+        <v>R$ 6999</v>
+      </c>
+      <c r="E59" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Protetor para Colchão Lençol Impermeável Matelado Com Toque Silencioso</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.2)</v>
+      </c>
+      <c r="C60" t="str">
+        <v>https://s.shopee.com.br/Ljg9D4Z8v</v>
+      </c>
+      <c r="D60" t="str">
+        <v>R$ 1490</v>
+      </c>
+      <c r="E60" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Carregador Portátil Mini Power Bank 10000mAh Com 02 Saídas Tipo-C / Lightning</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.34)</v>
+      </c>
+      <c r="C61" t="str">
+        <v>https://s.shopee.com.br/BQFwu5CTu</v>
+      </c>
+      <c r="D61" t="str">
+        <v>R$ 3199</v>
+      </c>
+      <c r="E61" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Gel Dental Pro White Hinode 90g</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.28)</v>
+      </c>
+      <c r="C62" t="str">
+        <v>https://s.shopee.com.br/16pkb5pot</v>
+      </c>
+      <c r="D62" t="str">
+        <v>R$ 1690</v>
+      </c>
+      <c r="E62" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2 Pcs Meias De Silicone Para O Cuidado Dos Pés Gel Hidratante Anti-Rachaduras Removedor De Pele Morta</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C63" t="str">
+        <v>https://s.shopee.com.br/2VoAjBwJkO</v>
+      </c>
+      <c r="D63" t="str">
+        <v>R$ 999</v>
+      </c>
+      <c r="E63" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Ventilador de Mesa 40 cm 10 Pás com 3 Velocidades Ventisol Turbo 10</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.48)</v>
+      </c>
+      <c r="C64" t="str">
+        <v>https://s.shopee.com.br/2LUkWswx5N</v>
+      </c>
+      <c r="D64" t="str">
+        <v>R$ 14990</v>
+      </c>
+      <c r="E64" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F64" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Extensão cabo PP Eletrica 50 Metros Reforçada Profissional 10/20a</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C65" t="str">
+        <v>https://s.shopee.com.br/2BBKKZxaQM</v>
+      </c>
+      <c r="D65" t="str">
+        <v>R$ 4900</v>
+      </c>
+      <c r="E65" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F65" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Copo Garrafa Térmica Grande Em Aço Inox Com Alça E Canudo Metal 1200ML</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.34)</v>
+      </c>
+      <c r="C66" t="str">
+        <v>https://s.shopee.com.br/20ru8GyDlL</v>
+      </c>
+      <c r="D66" t="str">
+        <v>R$ 3699</v>
+      </c>
+      <c r="E66" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F66" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Cueiro Estampado Flanelado Bebê Kit 3 Unidades 80X50CM Papi/Incomfral</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C67" t="str">
+        <v>https://s.shopee.com.br/1qYTvxyr6K</v>
+      </c>
+      <c r="D67" t="str">
+        <v>R$ 1999</v>
+      </c>
+      <c r="E67" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Garrafa Inox Térmica Com Capinha Protetora De Silicone Antiderrapante 1000ML</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.34)</v>
+      </c>
+      <c r="C68" t="str">
+        <v>https://s.shopee.com.br/1gF3jezURJ</v>
+      </c>
+      <c r="D68" t="str">
+        <v>R$ 3399</v>
+      </c>
+      <c r="E68" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F68" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>5/10/15/20 Metros Adesivo Papel de Parede Autocolante 5m x 45cm Madeira Mármore Geométrico 2,25m² Y2</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C69" t="str">
+        <v>https://s.shopee.com.br/1VvdXM07mI</v>
+      </c>
+      <c r="D69" t="str">
+        <v>R$ 1399</v>
+      </c>
+      <c r="E69" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Cesto Pão Porta Pães Bolacha Biscoito Organizador MDF Retrátil Cozinha Armazenamento</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C70" t="str">
+        <v>https://s.shopee.com.br/1LcDL30l7H</v>
+      </c>
+      <c r="D70" t="str">
+        <v>R$ 2800</v>
+      </c>
+      <c r="E70" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>46 Peças Verde Kit Chaves Jogo Catraca Reversível Soquetes Maleta Promoção</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
+      </c>
+      <c r="C71" t="str">
+        <v>https://s.shopee.com.br/3qJYJdrF2m</v>
+      </c>
+      <c r="D71" t="str">
+        <v>R$ 3099</v>
+      </c>
+      <c r="E71" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Kit Espátula Desencravador Slim Podologia - 3 Peças N206, N214 e Formão N254</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
+      </c>
+      <c r="C72" t="str">
+        <v>https://s.shopee.com.br/3g087KrsNl</v>
+      </c>
+      <c r="D72" t="str">
+        <v>R$ 1399</v>
+      </c>
+      <c r="E72" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F72" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Kit 5 Toalha de Banho Maldivas 100% algodão 60x120cm Sortidas</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.25)</v>
+      </c>
+      <c r="C73" t="str">
+        <v>https://s.shopee.com.br/3Vghv1sVik</v>
+      </c>
+      <c r="D73" t="str">
+        <v>R$ 5445</v>
+      </c>
+      <c r="E73" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F73" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>40/46 Peças Verde Kit Chaves Jogo Catraca Reversível Soquetes Maleta Promoção promoção</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
+      </c>
+      <c r="C74" t="str">
+        <v>https://s.shopee.com.br/3LNHiit93j</v>
+      </c>
+      <c r="D74" t="str">
+        <v>R$ 3099</v>
+      </c>
+      <c r="E74" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F74" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>The Perfect Top Insider</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
+      </c>
+      <c r="C75" t="str">
+        <v>https://s.shopee.com.br/3B3rWPtmOi</v>
+      </c>
+      <c r="D75" t="str">
+        <v>R$ 13500</v>
+      </c>
+      <c r="E75" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F75" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Cortina Blackout PVC Voil Xadrez 1,40 × 1,70 / 2,00 X 1,40</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.15)</v>
+      </c>
+      <c r="C76" t="str">
+        <v>https://s.shopee.com.br/30kRK6uPjh</v>
+      </c>
+      <c r="D76" t="str">
+        <v>R$ 3696</v>
+      </c>
+      <c r="E76" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F76" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>vestido  midi  de bolso  tamanho  único  g ,veste do 40 só 44, tecido  visco laycra</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.22)</v>
+      </c>
+      <c r="C77" t="str">
+        <v>https://s.shopee.com.br/2qR17nv34g</v>
+      </c>
+      <c r="D77" t="str">
+        <v>R$ 2699</v>
+      </c>
+      <c r="E77" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F77" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Toalha de Mesa Plástico Térmica Impermeável Premium para Mesas 4 CadeiraS / 6 Cadeiras / 8 Cadeiras</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C78" t="str">
+        <v>https://s.shopee.com.br/2g7avUvgPf</v>
+      </c>
+      <c r="D78" t="str">
+        <v>R$ 1196</v>
+      </c>
+      <c r="E78" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F78" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Papel Descartável Air Fryer Antiaderente Para Cozimento 50 Unidades</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.19)</v>
+      </c>
+      <c r="C79" t="str">
+        <v>https://s.shopee.com.br/5Aovu5mALA</v>
+      </c>
+      <c r="D79" t="str">
+        <v>R$ 1439</v>
+      </c>
+      <c r="E79" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F79" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Prateleira multiuso 4 andares modular.</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.17)</v>
+      </c>
+      <c r="C80" t="str">
+        <v>https://s.shopee.com.br/50VVhmmng9</v>
+      </c>
+      <c r="D80" t="str">
+        <v>R$ 2999</v>
+      </c>
+      <c r="E80" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F80" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Kit Completo p/ Projetor HY320 Mini – Com Suportes e Tampa de Lente - pronto par instalar</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.15)</v>
+      </c>
+      <c r="C81" t="str">
+        <v>https://s.shopee.com.br/4qC5VTnR18</v>
+      </c>
+      <c r="D81" t="str">
+        <v>R$ 3399</v>
+      </c>
+      <c r="E81" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F81" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Bebedouro Automatico Pet Fonte para Cães e Gatos Silenciosa Bivolt 1,5L</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.19)</v>
+      </c>
+      <c r="C82" t="str">
+        <v>https://s.shopee.com.br/4fsfJAo4M7</v>
+      </c>
+      <c r="D82" t="str">
+        <v>R$ 4899</v>
+      </c>
+      <c r="E82" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F82" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>QUEIMA DE ESTOQUE Tênis Feminino F1 Branco Casual Barato Do 34 ao 43 Masculino</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.19)</v>
+      </c>
+      <c r="C83" t="str">
+        <v>https://s.shopee.com.br/4VZF6rohh6</v>
+      </c>
+      <c r="D83" t="str">
+        <v>R$ 14990</v>
+      </c>
+      <c r="E83" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F83" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Kit 5 Cuecas Boxer Sandrini Algodão Adulto Masculinas Elastano Original cueca box Promoção</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.19)</v>
+      </c>
+      <c r="C84" t="str">
+        <v>https://s.shopee.com.br/4LFouYpL25</v>
+      </c>
+      <c r="D84" t="str">
+        <v>R$ 2499</v>
+      </c>
+      <c r="E84" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F84" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Caixa Caixinha De Som Bluetooth Potente Pendrive Fm Sd Portátil Ipx6</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
+      </c>
+      <c r="C85" t="str">
+        <v>https://s.shopee.com.br/4AwOiFpyN4</v>
+      </c>
+      <c r="D85" t="str">
+        <v>R$ 5500</v>
+      </c>
+      <c r="E85" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F85" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Microfone Lapela Sem Fio Duplo Kaidi Profissional Portátil Imã Redondo Anti Ruído Tipo C iPhone Gravação Celular</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.21)</v>
+      </c>
+      <c r="C86" t="str">
+        <v>https://s.shopee.com.br/40cyVwqbi3</v>
+      </c>
+      <c r="D86" t="str">
+        <v>R$ 7480</v>
+      </c>
+      <c r="E86" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F86" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Caixa de Som Grande Amplificada 2000w com Rodinha e 2 Microfones Sem Fio LED MP3</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.28)</v>
+      </c>
+      <c r="C87" t="str">
+        <v>https://s.shopee.com.br/6VKJUXh5dY</v>
+      </c>
+      <c r="D87" t="str">
+        <v>R$ 53199</v>
+      </c>
+      <c r="E87" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F87" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Fone De Ouvido Bluetooth Sem Fio I12 Touch Original Earphone TWS Anatel</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C88" t="str">
+        <v>https://s.shopee.com.br/6L0tIEhiyX</v>
+      </c>
+      <c r="D88" t="str">
+        <v>R$ 4549</v>
+      </c>
+      <c r="E88" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F88" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Caixa de Som Portatil Amplificada 2 Altos Falantes Caixinha Grande Potencia Heruz LED Bluetooth Recarregavel</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.33)</v>
+      </c>
+      <c r="C89" t="str">
+        <v>https://s.shopee.com.br/6AhT5viMJW</v>
+      </c>
+      <c r="D89" t="str">
+        <v>R$ 16399</v>
+      </c>
+      <c r="E89" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F89" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Fone de Ouvido Gamer Com Fio Headset Microfone Controle de Volume Original Inova</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.33)</v>
+      </c>
+      <c r="C90" t="str">
+        <v>https://s.shopee.com.br/60O2tcizeV</v>
+      </c>
+      <c r="D90" t="str">
+        <v>R$ 5890</v>
+      </c>
+      <c r="E90" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F90" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>CAIXA DE SOM PC GAMER COMPUTADOR KNUP HÓRUS R0850 – MULTIMÍDIA 2.0 | LED COLORIDO | 10W RMS | P2 + USB | WINDOWS / MAC</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.33)</v>
+      </c>
+      <c r="C91" t="str">
+        <v>https://s.shopee.com.br/5q4chJjczU</v>
+      </c>
+      <c r="D91" t="str">
+        <v>R$ 7499</v>
+      </c>
+      <c r="E91" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F91" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Fone de Ouvido Bluetooth Headphone Sem Fio Inova Original Graves Potentes</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.23)</v>
+      </c>
+      <c r="C92" t="str">
+        <v>https://s.shopee.com.br/5flCV0kGKT</v>
+      </c>
+      <c r="D92" t="str">
+        <v>R$ 7990</v>
+      </c>
+      <c r="E92" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F92" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Caixinha De Som Caixa Grande Potencia Led Bluetooth 2 Alto Falantes Heruz MP3</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.33)</v>
+      </c>
+      <c r="C93" t="str">
+        <v>https://s.shopee.com.br/5VRmIhktfS</v>
+      </c>
+      <c r="D93" t="str">
+        <v>R$ 15899</v>
+      </c>
+      <c r="E93" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F93" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Caixa de som Bluetooth Caixinha Grande Com Led RGB Portátil USB 2 Alto Falantes</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.33)</v>
+      </c>
+      <c r="C94" t="str">
+        <v>https://s.shopee.com.br/5L8M6OlX0R</v>
+      </c>
+      <c r="D94" t="str">
+        <v>R$ 15899</v>
+      </c>
+      <c r="E94" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F94" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Fone de Ouvido - Bluetooth - Sem Fio - Inova - IPhone - Android - Pequeno - Minimalista</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C95" t="str">
+        <v>https://s.shopee.com.br/7pph4zc0vw</v>
+      </c>
+      <c r="D95" t="str">
+        <v>R$ 5300</v>
+      </c>
+      <c r="E95" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F95" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Kit 3 Blusas Feminina Cores Brasil Copa Gola Alta Canelada Manga Curta Elegante Confortável</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.22)</v>
+      </c>
+      <c r="C96" t="str">
+        <v>https://s.shopee.com.br/7fWGsgceGv</v>
+      </c>
+      <c r="D96" t="str">
+        <v>R$ 4790</v>
+      </c>
+      <c r="E96" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F96" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>SAIA FEMININA COURO MIDI ENVELOPE AMARRAÇÃO + MODA SOCIAL</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C97" t="str">
+        <v>https://s.shopee.com.br/7VCqgNdHbu</v>
+      </c>
+      <c r="D97" t="str">
+        <v>R$ 7558</v>
+      </c>
+      <c r="E97" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F97" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Blusa Feminina Brasil T-shirt Verão Algodão</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.28)</v>
+      </c>
+      <c r="C98" t="str">
+        <v>https://s.shopee.com.br/7KtQU4duwt</v>
+      </c>
+      <c r="D98" t="str">
+        <v>R$ 3196</v>
+      </c>
+      <c r="E98" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F98" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Conjuntos de manga longa em torno do pescoço impresso moletom e leggings</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.18)</v>
+      </c>
+      <c r="C99" t="str">
+        <v>https://s.shopee.com.br/7Aa0HleYHs</v>
+      </c>
+      <c r="D99" t="str">
+        <v>R$ 9833</v>
+      </c>
+      <c r="E99" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F99" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Kit pijama mãe e filha capivara inverno calça estampada malha blusa manga comprida personagens inverno frio longo</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.21)</v>
+      </c>
+      <c r="C100" t="str">
+        <v>https://s.shopee.com.br/70Ga5SfBcr</v>
+      </c>
+      <c r="D100" t="str">
+        <v>R$ 7920</v>
+      </c>
+      <c r="E100" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F100" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Cropped Top Feminino Alcinha Frente Forrada Personalizado Copa 2026 ESTHER BRASIL</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Oferta Especial Shopee (Comissão: 0.2)</v>
+      </c>
+      <c r="C101" t="str">
+        <v>https://s.shopee.com.br/6px9t9foxq</v>
+      </c>
+      <c r="D101" t="str">
+        <v>R$ 2983</v>
+      </c>
+      <c r="E101" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/f/fe/Shopee.svg/256px-Shopee.svg.png</v>
+      </c>
+      <c r="F101" t="str">
         <v>Shopee</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F101"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Integracao de links do OneDrive com imagens reais capturadas
</commit_message>
<xml_diff>
--- a/shopee.xlsx
+++ b/shopee.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Produtos" sheetId="1" r:id="rId1"/>
+    <sheet name="Links OneDrive" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,16 +424,16 @@
         <v>40 Peças / 46 Peças Jogo De Chave Catraca Caixa De Ferramentas Completa Reversível Soquetes Maleta</v>
       </c>
       <c r="B2" t="str">
-        <v>Oferta Shopee (0.19)</v>
+        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
       </c>
       <c r="C2" t="str">
         <v>https://s.shopee.com.br/2BBKKZxaPL</v>
       </c>
       <c r="D2" t="str">
-        <v>R$ 30,99</v>
+        <v>R$ 30,99</v>
       </c>
       <c r="E2" t="str">
-        <v>https://m.media-amazon.com/images/I/71z+6P8f6NL._AC_SL1500_.jpg</v>
+        <v>https://m.media-amazon.com/images/I/81MzIgh8luL.jpg</v>
       </c>
       <c r="F2" t="str">
         <v>Shopee</v>
@@ -441,27 +441,187 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>Kit Collagen Completo Máscara 500g Shampoo 1L Condicionador 1L Óleo Maca 50ml Tratamento Profissional</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>https://s.shopee.com.br/1gf3jezUQG</v>
+      </c>
+      <c r="D3" t="str">
+        <v>R$ 54,00</v>
+      </c>
+      <c r="E3" t="str">
+        <v>https://down-br.img.susercontent.com/file/br-11134207-820m4-mnb6ge4ki9dt70</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
         <v>Jogo de Lençol 400 Fios Cama Solteiro Casal Queen King E Berço Micropercal Ponto Palito</v>
       </c>
-      <c r="B3" t="str">
-        <v>Oferta Shopee (0.21)</v>
-      </c>
-      <c r="C3" t="str">
-        <v>https://s.shopee.com.br/1qYTvxyr5J</v>
-      </c>
-      <c r="D3" t="str">
-        <v>R$ 27,23</v>
-      </c>
-      <c r="E3" t="str">
-        <v>https://m.media-amazon.com/images/I/61N6N6N6N6L._AC_SL1000_.jpg</v>
-      </c>
-      <c r="F3" t="str">
+      <c r="B4" t="str">
+        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>https://s.shopee.com.br/1qYTxvyr5J</v>
+      </c>
+      <c r="D4" t="str">
+        <v>R$ 27,23</v>
+      </c>
+      <c r="E4" t="str">
+        <v>https://down-br.img.susercontent.com/file/br-11134207-7qukw-ljj75v06g0i857</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Kit 1 ou 2 Unidades de Veda Porta Ajustável Protetor Rolinho Impermeável 80cm 90cm 100cm</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>https://s.shopee.com.br/1LcDL30l6E</v>
+      </c>
+      <c r="D5" t="str">
+        <v>R$ 12,54</v>
+      </c>
+      <c r="E5" t="str">
+        <v>https://m.media-amazon.com/images/I/51WhpiChLTL.jpg</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Kit Limpador Pastilha de máquina de lavar roupa, comprimido efervescente sólido para remover manchas</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>https://s.shopee.com.br/1VvdXM07IH</v>
+      </c>
+      <c r="D6" t="str">
+        <v>R$ 8,59</v>
+      </c>
+      <c r="E6" t="str">
+        <v>https://m.media-amazon.com/images/I/71MghNSCDPL._AC_UF1000,1000_QL80_.jpg</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Kit 3 Peneira Coador De Peneiras Aço Inoxidável Para Cozinha Peneira De Cozinha</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>https://s.shopee.com.br/3g087KrsMi</v>
+      </c>
+      <c r="D7" t="str">
+        <v>R$ 15,99</v>
+      </c>
+      <c r="E7" t="str">
+        <v>https://m.media-amazon.com/images/I/71A3ImQhfHL._AC_UF894,1000_QL80_.jpg</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Inox Torneira Prata/Preto Com Chuveiro Com Rotação De 360° Cozinha Luxo Parede Promoção</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>https://s.shopee.com.br/3qJYJdrF1l</v>
+      </c>
+      <c r="D8" t="str">
+        <v>R$ 23,99</v>
+      </c>
+      <c r="E8" t="str">
+        <v>https://down-br.img.susercontent.com/file/br-11134207-820mb-mlx7ds1np5omf4</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Kit 1/2/5 Suporte De Parede Multifuncional Caixa De Armazenamento Casa Para Carregar Remoto Um Slot Promoção</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>https://s.shopee.com.br/3LNHIit92g</v>
+      </c>
+      <c r="D9" t="str">
+        <v>R$ 9,59</v>
+      </c>
+      <c r="E9" t="str">
+        <v>https://down-br.img.susercontent.com/file/br-11134207-7qukw-ljpumel2dxmy85</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Mangueira de Jardim Anti-Torção e Anti-Dobras de 5 a 50 Metros</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>https://s.shopee.com.br/3Vghv1sVhj</v>
+      </c>
+      <c r="D10" t="str">
+        <v>R$ 17,32</v>
+      </c>
+      <c r="E10" t="str">
+        <v>https://down-br.img.susercontent.com/file/br-11134207-7r98o-m4zac7gestxh75</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Creme Desodorante Antitranspirante Herbíssimo Care Rosa Mosqueta E Niacinamida Bisnaga 55g</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+      </c>
+      <c r="C11" t="str">
+        <v>https://s.shopee.com.br/30kRK6uPie</v>
+      </c>
+      <c r="D11" t="str">
+        <v>R$ 16,99</v>
+      </c>
+      <c r="E11" t="str">
+        <v>https://epocacosmeticos.vteximg.com.br/arquivos/ids/792015-800-800/17404927504767.jpg?v=638772260539870000</v>
+      </c>
+      <c r="F11" t="str">
         <v>Shopee</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Upload de todos os 100 links de afiliados do CSV e melhoria no UI Fallback
</commit_message>
<xml_diff>
--- a/shopee.xlsx
+++ b/shopee.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Links OneDrive" sheetId="1" r:id="rId1"/>
+    <sheet name="Produtos" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F101"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,16 +424,16 @@
         <v>40 Peças / 46 Peças Jogo De Chave Catraca Caixa De Ferramentas Completa Reversível Soquetes Maleta</v>
       </c>
       <c r="B2" t="str">
-        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+        <v>Oferta Especial Shopee (0.19)</v>
       </c>
       <c r="C2" t="str">
         <v>https://s.shopee.com.br/2BBKKZxaPL</v>
       </c>
       <c r="D2" t="str">
-        <v>R$ 30,99</v>
+        <v>R$ 30,99</v>
       </c>
       <c r="E2" t="str">
-        <v>https://m.media-amazon.com/images/I/81MzIgh8luL.jpg</v>
+        <v/>
       </c>
       <c r="F2" t="str">
         <v>Shopee</v>
@@ -441,19 +441,19 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Kit Collagen Completo Máscara 500g Shampoo 1L Condicionador 1L Óleo Maca 50ml Tratamento Profissional</v>
+        <v>Kit  Collagen Completo Máscara 500g Shampoo 1L Condicionador 1L Óleo Maca 50ml Tratamento Profissional</v>
       </c>
       <c r="B3" t="str">
-        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+        <v>Oferta Especial Shopee (0.16)</v>
       </c>
       <c r="C3" t="str">
-        <v>https://s.shopee.com.br/1gf3jezUQG</v>
+        <v>https://s.shopee.com.br/1gF3jezUQG</v>
       </c>
       <c r="D3" t="str">
-        <v>R$ 54,00</v>
+        <v>R$ 54,00</v>
       </c>
       <c r="E3" t="str">
-        <v>https://down-br.img.susercontent.com/file/br-11134207-820m4-mnb6ge4ki9dt70</v>
+        <v/>
       </c>
       <c r="F3" t="str">
         <v>Shopee</v>
@@ -464,16 +464,16 @@
         <v>Jogo de Lençol 400 Fios Cama Solteiro Casal Queen King E Berço Micropercal Ponto Palito</v>
       </c>
       <c r="B4" t="str">
-        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+        <v>Oferta Especial Shopee (0.21)</v>
       </c>
       <c r="C4" t="str">
-        <v>https://s.shopee.com.br/1qYTxvyr5J</v>
+        <v>https://s.shopee.com.br/1qYTvxyr5J</v>
       </c>
       <c r="D4" t="str">
-        <v>R$ 27,23</v>
+        <v>R$ 27,23</v>
       </c>
       <c r="E4" t="str">
-        <v>https://down-br.img.susercontent.com/file/br-11134207-7qukw-ljj75v06g0i857</v>
+        <v/>
       </c>
       <c r="F4" t="str">
         <v>Shopee</v>
@@ -484,16 +484,16 @@
         <v>Kit 1 ou 2 Unidades de Veda Porta Ajustável Protetor Rolinho Impermeável 80cm 90cm 100cm</v>
       </c>
       <c r="B5" t="str">
-        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+        <v>Oferta Especial Shopee (0.24)</v>
       </c>
       <c r="C5" t="str">
         <v>https://s.shopee.com.br/1LcDL30l6E</v>
       </c>
       <c r="D5" t="str">
-        <v>R$ 12,54</v>
+        <v>R$ 12,54</v>
       </c>
       <c r="E5" t="str">
-        <v>https://m.media-amazon.com/images/I/51WhpiChLTL.jpg</v>
+        <v/>
       </c>
       <c r="F5" t="str">
         <v>Shopee</v>
@@ -501,19 +501,19 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Kit Limpador Pastilha de máquina de lavar roupa, comprimido efervescente sólido para remover manchas</v>
+        <v>Kit Limpador Pastilha de máquina de lavar roupa, comprimido efervescente sólido para remover manchas【】</v>
       </c>
       <c r="B6" t="str">
-        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+        <v>Oferta Especial Shopee (0.18)</v>
       </c>
       <c r="C6" t="str">
-        <v>https://s.shopee.com.br/1VvdXM07IH</v>
+        <v>https://s.shopee.com.br/1VvdXM07lH</v>
       </c>
       <c r="D6" t="str">
-        <v>R$ 8,59</v>
+        <v>R$ 859,00</v>
       </c>
       <c r="E6" t="str">
-        <v>https://m.media-amazon.com/images/I/71MghNSCDPL._AC_UF1000,1000_QL80_.jpg</v>
+        <v/>
       </c>
       <c r="F6" t="str">
         <v>Shopee</v>
@@ -524,16 +524,16 @@
         <v>Kit 3 Peneira Coador De Peneiras Aço Inoxidável Para Cozinha Peneira De Cozinha</v>
       </c>
       <c r="B7" t="str">
-        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+        <v>Oferta Especial Shopee (0.15)</v>
       </c>
       <c r="C7" t="str">
         <v>https://s.shopee.com.br/3g087KrsMi</v>
       </c>
       <c r="D7" t="str">
-        <v>R$ 15,99</v>
+        <v>R$ 15,99</v>
       </c>
       <c r="E7" t="str">
-        <v>https://m.media-amazon.com/images/I/71A3ImQhfHL._AC_UF894,1000_QL80_.jpg</v>
+        <v/>
       </c>
       <c r="F7" t="str">
         <v>Shopee</v>
@@ -541,19 +541,19 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Inox Torneira Prata/Preto Com Chuveiro Com Rotação De 360° Cozinha Luxo Parede Promoção</v>
+        <v>Inox Torneira  Prata/Preto Com Chuveiro Com Rotação De 360° Cozinha Luxo Parede Promoção</v>
       </c>
       <c r="B8" t="str">
-        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+        <v>Oferta Especial Shopee (0.23)</v>
       </c>
       <c r="C8" t="str">
         <v>https://s.shopee.com.br/3qJYJdrF1l</v>
       </c>
       <c r="D8" t="str">
-        <v>R$ 23,99</v>
+        <v>R$ 23,99</v>
       </c>
       <c r="E8" t="str">
-        <v>https://down-br.img.susercontent.com/file/br-11134207-820mb-mlx7ds1np5omf4</v>
+        <v/>
       </c>
       <c r="F8" t="str">
         <v>Shopee</v>
@@ -561,19 +561,19 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Kit 1/2/5 Suporte De Parede Multifuncional Caixa De Armazenamento Casa Para Carregar Remoto Um Slot Promoção</v>
+        <v>KIT 1/2/5 Suporte De Parede Multifuncional Caixa De Armazenamento Casa Para Carregar Remoto Um Slot Promoção</v>
       </c>
       <c r="B9" t="str">
-        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+        <v>Oferta Especial Shopee (0.23)</v>
       </c>
       <c r="C9" t="str">
-        <v>https://s.shopee.com.br/3LNHIit92g</v>
+        <v>https://s.shopee.com.br/3LNHiit92g</v>
       </c>
       <c r="D9" t="str">
-        <v>R$ 9,59</v>
+        <v>R$ 959,00</v>
       </c>
       <c r="E9" t="str">
-        <v>https://down-br.img.susercontent.com/file/br-11134207-7qukw-ljpumel2dxmy85</v>
+        <v/>
       </c>
       <c r="F9" t="str">
         <v>Shopee</v>
@@ -584,16 +584,16 @@
         <v>Mangueira de Jardim Anti-Torção e Anti-Dobras de 5 a 50 Metros</v>
       </c>
       <c r="B10" t="str">
-        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+        <v>Oferta Especial Shopee (0.21)</v>
       </c>
       <c r="C10" t="str">
         <v>https://s.shopee.com.br/3Vghv1sVhj</v>
       </c>
       <c r="D10" t="str">
-        <v>R$ 17,32</v>
+        <v>R$ 17,32</v>
       </c>
       <c r="E10" t="str">
-        <v>https://down-br.img.susercontent.com/file/br-11134207-7r98o-m4zac7gestxh75</v>
+        <v/>
       </c>
       <c r="F10" t="str">
         <v>Shopee</v>
@@ -604,24 +604,1824 @@
         <v>Creme Desodorante Antitranspirante Herbíssimo Care Rosa Mosqueta E Niacinamida Bisnaga 55g</v>
       </c>
       <c r="B11" t="str">
-        <v>Oferta Especial Shopee (Visto no OneDrive)</v>
+        <v>Oferta Especial Shopee (0.17)</v>
       </c>
       <c r="C11" t="str">
         <v>https://s.shopee.com.br/30kRK6uPie</v>
       </c>
       <c r="D11" t="str">
-        <v>R$ 16,99</v>
+        <v>R$ 16,99</v>
       </c>
       <c r="E11" t="str">
-        <v>https://epocacosmeticos.vteximg.com.br/arquivos/ids/792015-800-800/17404927504767.jpg?v=638772260539870000</v>
+        <v/>
       </c>
       <c r="F11" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Kit Maca Power Completo com 7 Produtos – Cronograma Capilar + Máscara 500g, Shampoo 1L, Condicionador 1L  Reparador 50ml</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Oferta Especial Shopee (0.16)</v>
+      </c>
+      <c r="C12" t="str">
+        <v>https://s.shopee.com.br/3B3rWPtmNh</v>
+      </c>
+      <c r="D12" t="str">
+        <v>R$ 78,00</v>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Creme Depilatório Corporal Depilsam Aloe Vera 200G</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Oferta Especial Shopee (0.17)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>https://s.shopee.com.br/2g7avUvgOc</v>
+      </c>
+      <c r="D13" t="str">
+        <v>R$ 24,98</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Protetor de Colchão Impermeável Matelado Varias Cores Para Cama Box Solteiro, Casal, Queen, King, Mini Berço E Berço</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Oferta Especial Shopee (0.24)</v>
+      </c>
+      <c r="C14" t="str">
+        <v>https://s.shopee.com.br/2qR17nv33f</v>
+      </c>
+      <c r="D14" t="str">
+        <v>R$ 15,90</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>KIT 3, 6 e 9 Calcinha Feminina Tanga Infantil Juvenil Algodão Macio Ajuste Perfeito Cores Estampas Sortidas</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C15" t="str">
+        <v>https://s.shopee.com.br/50VVhmmnf6</v>
+      </c>
+      <c r="D15" t="str">
+        <v>R$ 15,90</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>JBSARA Soro Renovador de Retinol 1ml Envio da Coreia 1 peça</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>https://s.shopee.com.br/5Aovu5mAK9</v>
+      </c>
+      <c r="D16" t="str">
+        <v>R$ 349,00</v>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Regata Alça Fina Fitness Blusa Feminino Liso Poliamida Tank Top Slim Camiseta Academia Verão</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>https://s.shopee.com.br/4fsfJAo4L4</v>
+      </c>
+      <c r="D17" t="str">
+        <v>R$ 37,90</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Fórmula de Lyah 60 doses - Suplemento Alimentar</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Oferta Especial Shopee (0.25)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>https://s.shopee.com.br/4qC5VTnR07</v>
+      </c>
+      <c r="D18" t="str">
+        <v>R$ 69,90</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Creme Gel Regenerador Facial Gota de Colágeno Kokeshi 45g</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Oferta Especial Shopee (0.24)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>https://s.shopee.com.br/4LFouYpL12</v>
+      </c>
+      <c r="D19" t="str">
+        <v>R$ 32,83</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Creme Para Pentear Definição Natural 1kg</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>https://s.shopee.com.br/4VZF6rohg5</v>
+      </c>
+      <c r="D20" t="str">
+        <v>R$ 35,75</v>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Cinta Modeladora Espartilho De Emagrecimento-ENVIO IMEDIATO --8888</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Oferta Especial Shopee (0.16)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>https://s.shopee.com.br/40cyVwqbh0</v>
+      </c>
+      <c r="D21" t="str">
+        <v>R$ 22,80</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>1/2/3 Forro Antiderrapante Para Gaveta, Geladeira E Guarda Roupas- Transparente 0,6*3M Evita Deslizamento em Superfícies</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C22" t="str">
+        <v>https://s.shopee.com.br/4AwOiFpyM3</v>
+      </c>
+      <c r="D22" t="str">
+        <v>R$ 23,99</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Kit 10 Marmita conjunto Potes 750ml com Travas Laterais BPA FREE - Alimentos organizadores de congelador</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>https://s.shopee.com.br/6L0tIEhixU</v>
+      </c>
+      <c r="D23" t="str">
+        <v>R$ 21,90</v>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Relógio Masculino digital wr | 100 % qualidade | entrega rápida</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>https://s.shopee.com.br/6VKJUXh5cX</v>
+      </c>
+      <c r="D24" t="str">
+        <v>R$ 12,99</v>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Coberdrom Cobertor Solteiro Casal Queen E King Colcha Dupla Face Edredrom Luxo Pele Carneiro Premium</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>https://s.shopee.com.br/60O2tcizdS</v>
+      </c>
+      <c r="D25" t="str">
+        <v>R$ 94,98</v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Amplificador De Imagem Da Tela Do Celular Lupa 3D 21,6CM*16,6CM*2,7CM Promoção</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>https://s.shopee.com.br/6AhT5viMIV</v>
+      </c>
+      <c r="D26" t="str">
+        <v>R$ 17,99</v>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Óleo de Tratamento SOS Cachos 10 em 1 Multibenefícios 42ml</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>https://s.shopee.com.br/5flCV0kGJQ</v>
+      </c>
+      <c r="D27" t="str">
+        <v>R$ 16,20</v>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Arranjo c/ 3 Trepadeira Folha de HERA + Vaso Trançado Marrom</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Oferta Especial Shopee (0.28)</v>
+      </c>
+      <c r="C28" t="str">
+        <v>https://s.shopee.com.br/5q4chJjcyT</v>
+      </c>
+      <c r="D28" t="str">
+        <v>R$ 16,80</v>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Alvejante Poderoso com Percarbonato de Sódio Tira Manchas Roupas Brancas e Coloridas -GF Agro</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Oferta Especial Shopee (0.22)</v>
+      </c>
+      <c r="C29" t="str">
+        <v>https://s.shopee.com.br/5L8M6OlWzO</v>
+      </c>
+      <c r="D29" t="str">
+        <v>R$ 11,99</v>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>30 unidades cabide redondo resistente adulto</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Oferta Especial Shopee (0.17)</v>
+      </c>
+      <c r="C30" t="str">
+        <v>https://s.shopee.com.br/5VRmIhkteR</v>
+      </c>
+      <c r="D30" t="str">
+        <v>R$ 19,98</v>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Principia Kit Completo Peles Sensíveis c/ Gel de Limpeza Gl-02 + Creme Hidratante CH-01 + Protetor Solar PS-01 FPS 60</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C31" t="str">
+        <v>https://s.shopee.com.br/7fWGsgceFs</v>
+      </c>
+      <c r="D31" t="str">
+        <v>R$ 116,25</v>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+      <c r="F31" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Cera Espelhamento RENOVE – Remove Riscos Superficiais, Repele Água, Proteção Sol, Brilho Intenso</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Oferta Especial Shopee (0.24)</v>
+      </c>
+      <c r="C32" t="str">
+        <v>https://s.shopee.com.br/7pph4zc0uv</v>
+      </c>
+      <c r="D32" t="str">
+        <v>R$ 17,99</v>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Kit 10, 5 Cueca Masculina Box Adulto Microfibra Forro 100% Algodão Cores Variadas</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C33" t="str">
+        <v>https://s.shopee.com.br/7KtQU4duvq</v>
+      </c>
+      <c r="D33" t="str">
+        <v>R$ 26,80</v>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Mini Umidificador Difusor Aromatizador Egg Portátil Usb Led Aromatizador De Ambiente Purificador De Ar Casa Escritório</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C34" t="str">
+        <v>https://s.shopee.com.br/7VCqgNdHat</v>
+      </c>
+      <c r="D34" t="str">
+        <v>R$ 16,99</v>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Luminária Despertador Com Luz Led Bluetooth Caixa  Som Relógio Digital  Carregamento Indução Abajur</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C35" t="str">
+        <v>https://s.shopee.com.br/70Ga5SfBbo</v>
+      </c>
+      <c r="D35" t="str">
+        <v>R$ 34,90</v>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>kit Coala Home Chá Branco</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C36" t="str">
+        <v>https://s.shopee.com.br/7Aa0HleYGr</v>
+      </c>
+      <c r="D36" t="str">
+        <v>R$ 69,99</v>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Cafe Graos Torra Media Gourmet Café Italle 1kg</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Oferta Especial Shopee (0.28)</v>
+      </c>
+      <c r="C37" t="str">
+        <v>https://s.shopee.com.br/6fdjgqgSHm</v>
+      </c>
+      <c r="D37" t="str">
+        <v>R$ 71,30</v>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Cinto Masculino Feminino Tecido Trançado Elástico Fivela De Metal</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Oferta Especial Shopee (0.17)</v>
+      </c>
+      <c r="C38" t="str">
+        <v>https://s.shopee.com.br/6px9t9fowp</v>
+      </c>
+      <c r="D38" t="str">
+        <v>R$ 10,99</v>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Kit de 72 unidades de Xuxinha de cabelo elastico de para cabelo feminino rabicó</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C39" t="str">
+        <v>https://s.shopee.com.br/901eT8XZYG</v>
+      </c>
+      <c r="D39" t="str">
+        <v>R$ 10,87</v>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Manta Cobertor Microfibra Casal Queen King Quentinha Antialérgico Poá Habitat</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Oferta Especial Shopee (0.21)</v>
+      </c>
+      <c r="C40" t="str">
+        <v>https://s.shopee.com.br/9AL4fRWwDJ</v>
+      </c>
+      <c r="D40" t="str">
+        <v>R$ 52,89</v>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Pistola Elétrica Para Pintura Pulverizador de Tinta com Bico de Metal e Compressor 450w - TSSAPER</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C41" t="str">
+        <v>https://s.shopee.com.br/8fOo4WYqEE</v>
+      </c>
+      <c r="D41" t="str">
+        <v>R$ 137,45</v>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Lençol Com Elástico Premium Avulso 400 Fios Percal Liso Toque Macio Acetinado</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C42" t="str">
+        <v>https://s.shopee.com.br/8piEGpYCtH</v>
+      </c>
+      <c r="D42" t="str">
+        <v>R$ 18,80</v>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Balança Corporal Transparente Quadrada Digital Até 180kg Com Vidro Temperado Premium</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C43" t="str">
+        <v>https://s.shopee.com.br/8Klxfua6uC</v>
+      </c>
+      <c r="D43" t="str">
+        <v>R$ 32,99</v>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>2025 Nova Série 8 Relógio T800 Ultra Smart Watch Esportivo Sem Fio À Prova D'água T800 Ultra2 MAX</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Oferta Especial Shopee (0.16)</v>
+      </c>
+      <c r="C44" t="str">
+        <v>https://s.shopee.com.br/8V5NsDZTZF</v>
+      </c>
+      <c r="D44" t="str">
+        <v>R$ 38,99</v>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Protetor Solar Facial PS-01 FPS 60 Principia</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C45" t="str">
+        <v>https://s.shopee.com.br/8097HIbNaA</v>
+      </c>
+      <c r="D45" t="str">
+        <v>R$ 49,00</v>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+      <c r="F45" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Leggings canelada de cintura larga e cor sólida para atividades esportivas.</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C46" t="str">
+        <v>https://s.shopee.com.br/8ASXTbakFD</v>
+      </c>
+      <c r="D46" t="str">
+        <v>R$ 29,99</v>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Blusa Feminina Manga 3/4 Novas Cores Tecido Crepe Moda Evangelica Detalhe Social Elegante</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Oferta Especial Shopee (0.34)</v>
+      </c>
+      <c r="C47" t="str">
+        <v>https://s.shopee.com.br/AKX23aSUqe</v>
+      </c>
+      <c r="D47" t="str">
+        <v>R$ 26,99</v>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Fita Multiuso Manta Asfaltica Adesiva para Reparos Rufo Calha Telhado Veda Tudo 10cm 20cm 30cm POR METRO</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Oferta Especial Shopee (0.16)</v>
+      </c>
+      <c r="C48" t="str">
+        <v>https://s.shopee.com.br/AUqSFtRrVh</v>
+      </c>
+      <c r="D48" t="str">
+        <v>R$ 999,00</v>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Blusa Manga 3/4 Detalhe Em V Novas Cores Verão Tendência Moda Feminina</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Oferta Especial Shopee (0.17)</v>
+      </c>
+      <c r="C49" t="str">
+        <v>https://s.shopee.com.br/9zuBeyTlWc</v>
+      </c>
+      <c r="D49" t="str">
+        <v>R$ 26,99</v>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Kit M10 Bluetooth 5.3 Sem Fio TWS Fones De Ouvido Estéreo Com Carregador Power Bank Atualizado 100 % Novo Alto-Falante</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C50" t="str">
+        <v>https://s.shopee.com.br/AADbrHT8Bf</v>
+      </c>
+      <c r="D50" t="str">
+        <v>R$ 25,89</v>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Shampoo Tonalizante Escurecedor S/ Amônia Avelã, Marsala, Loiro, Vermelho Ruivo 100% Natural Matizze</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C51" t="str">
+        <v>https://s.shopee.com.br/9fHLGMV2Ca</v>
+      </c>
+      <c r="D51" t="str">
+        <v>R$ 17,89</v>
+      </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
+      <c r="F51" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Kit de Óleo Capilar - Cronograma Terapia Capilar - 100% natural - 60ml</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Oferta Especial Shopee (0.2)</v>
+      </c>
+      <c r="C52" t="str">
+        <v>https://s.shopee.com.br/9palSfUOrd</v>
+      </c>
+      <c r="D52" t="str">
+        <v>R$ 15,30</v>
+      </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
+      <c r="F52" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Carregador Portátil Mini Power Bank 10000mAh Com 02 Saídas Tipo-C / Lightning</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Oferta Especial Shopee (0.34)</v>
+      </c>
+      <c r="C53" t="str">
+        <v>https://s.shopee.com.br/9KeUrkWIsY</v>
+      </c>
+      <c r="D53" t="str">
+        <v>R$ 32,99</v>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+      <c r="F53" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Mini Barbeador Elétrico Portátil À Prova D'água De Dupla Finalidade Tipo c De Carga Rápida Aparador De Barba De Bolso</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C54" t="str">
+        <v>https://s.shopee.com.br/9Uxv43VfXb</v>
+      </c>
+      <c r="D54" t="str">
+        <v>R$ 16,99</v>
+      </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
+      <c r="F54" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Trava Óculos Antiderrapante Silicone Kit Não Cai Do Rosto Gancho Orelha Haste Conforto</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C55" t="str">
+        <v>https://s.shopee.com.br/1BIn8k1OS0</v>
+      </c>
+      <c r="D55" t="str">
+        <v>R$ 700,00</v>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Kit 3 Bermudas Masculina Esportivo Academia Praia Com  Bolsos E Refletivo</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C56" t="str">
+        <v>https://s.shopee.com.br/10zMwR21mz</v>
+      </c>
+      <c r="D56" t="str">
+        <v>R$ 44,04</v>
+      </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+      <c r="F56" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Kit Com 10 ou 4 Cuecas Boxers Premium Masculina Adulto de Microfibra</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C57" t="str">
+        <v>https://s.shopee.com.br/qfwk82f7y</v>
+      </c>
+      <c r="D57" t="str">
+        <v>R$ 24,98</v>
+      </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
+      <c r="F57" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Shorts modeladores sem costura com forro de microfibra</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Oferta Especial Shopee (0.16)</v>
+      </c>
+      <c r="C58" t="str">
+        <v>https://s.shopee.com.br/gMWXp3ISx</v>
+      </c>
+      <c r="D58" t="str">
+        <v>R$ 19,24</v>
+      </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
+      <c r="F58" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Kit 4pçs Toalhas de Banho 140x70cm 100% Algodão Premium Coleção Difiori</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C59" t="str">
+        <v>https://s.shopee.com.br/W36LW3vnw</v>
+      </c>
+      <c r="D59" t="str">
+        <v>R$ 69,99</v>
+      </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
+      <c r="F59" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Protetor para Colchão Lençol Impermeável Matelado Com Toque Silencioso</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Oferta Especial Shopee (0.2)</v>
+      </c>
+      <c r="C60" t="str">
+        <v>https://s.shopee.com.br/Ljg9D4Z8v</v>
+      </c>
+      <c r="D60" t="str">
+        <v>R$ 14,90</v>
+      </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
+      <c r="F60" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Carregador Portátil Mini Power Bank 10000mAh Com 02 Saídas Tipo-C / Lightning</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Oferta Especial Shopee (0.34)</v>
+      </c>
+      <c r="C61" t="str">
+        <v>https://s.shopee.com.br/BQFwu5CTu</v>
+      </c>
+      <c r="D61" t="str">
+        <v>R$ 31,99</v>
+      </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
+      <c r="F61" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Gel Dental Pro White Hinode 90g</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Oferta Especial Shopee (0.28)</v>
+      </c>
+      <c r="C62" t="str">
+        <v>https://s.shopee.com.br/16pkb5pot</v>
+      </c>
+      <c r="D62" t="str">
+        <v>R$ 16,90</v>
+      </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
+      <c r="F62" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2 Pcs Meias De Silicone Para O Cuidado Dos Pés Gel Hidratante Anti-Rachaduras Removedor De Pele Morta</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C63" t="str">
+        <v>https://s.shopee.com.br/2VoAjBwJkO</v>
+      </c>
+      <c r="D63" t="str">
+        <v>R$ 999,00</v>
+      </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
+      <c r="F63" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Ventilador de Mesa 40 cm 10 Pás com 3 Velocidades Ventisol Turbo 10</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Oferta Especial Shopee (0.48)</v>
+      </c>
+      <c r="C64" t="str">
+        <v>https://s.shopee.com.br/2LUkWswx5N</v>
+      </c>
+      <c r="D64" t="str">
+        <v>R$ 149,90</v>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+      <c r="F64" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Extensão cabo PP Eletrica 50 Metros Reforçada Profissional 10/20a</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C65" t="str">
+        <v>https://s.shopee.com.br/2BBKKZxaQM</v>
+      </c>
+      <c r="D65" t="str">
+        <v>R$ 49,00</v>
+      </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
+      <c r="F65" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Copo Garrafa Térmica Grande Em Aço Inox Com Alça E Canudo Metal 1200ML</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Oferta Especial Shopee (0.34)</v>
+      </c>
+      <c r="C66" t="str">
+        <v>https://s.shopee.com.br/20ru8GyDlL</v>
+      </c>
+      <c r="D66" t="str">
+        <v>R$ 36,99</v>
+      </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
+      <c r="F66" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Cueiro Estampado Flanelado Bebê Kit 3 Unidades 80X50CM Papi/Incomfral</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C67" t="str">
+        <v>https://s.shopee.com.br/1qYTvxyr6K</v>
+      </c>
+      <c r="D67" t="str">
+        <v>R$ 19,99</v>
+      </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
+      <c r="F67" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Garrafa Inox Térmica Com Capinha Protetora De Silicone Antiderrapante 1000ML</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Oferta Especial Shopee (0.34)</v>
+      </c>
+      <c r="C68" t="str">
+        <v>https://s.shopee.com.br/1gF3jezURJ</v>
+      </c>
+      <c r="D68" t="str">
+        <v>R$ 33,99</v>
+      </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
+      <c r="F68" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>5/10/15/20 Metros Adesivo Papel de Parede Autocolante 5m x 45cm Madeira Mármore Geométrico 2,25m² Y2</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C69" t="str">
+        <v>https://s.shopee.com.br/1VvdXM07mI</v>
+      </c>
+      <c r="D69" t="str">
+        <v>R$ 13,99</v>
+      </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
+      <c r="F69" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Cesto Pão Porta Pães Bolacha Biscoito Organizador MDF Retrátil Cozinha Armazenamento</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C70" t="str">
+        <v>https://s.shopee.com.br/1LcDL30l7H</v>
+      </c>
+      <c r="D70" t="str">
+        <v>R$ 28,00</v>
+      </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
+      <c r="F70" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>46 Peças Verde Kit Chaves Jogo Catraca Reversível Soquetes Maleta Promoção</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C71" t="str">
+        <v>https://s.shopee.com.br/3qJYJdrF2m</v>
+      </c>
+      <c r="D71" t="str">
+        <v>R$ 30,99</v>
+      </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
+      <c r="F71" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Kit Espátula Desencravador Slim Podologia - 3 Peças N206, N214 e Formão N254</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C72" t="str">
+        <v>https://s.shopee.com.br/3g087KrsNl</v>
+      </c>
+      <c r="D72" t="str">
+        <v>R$ 13,99</v>
+      </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
+      <c r="F72" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Kit 5 Toalha de Banho Maldivas 100% algodão 60x120cm Sortidas</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Oferta Especial Shopee (0.25)</v>
+      </c>
+      <c r="C73" t="str">
+        <v>https://s.shopee.com.br/3Vghv1sVik</v>
+      </c>
+      <c r="D73" t="str">
+        <v>R$ 54,45</v>
+      </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
+      <c r="F73" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>40/46 Peças Verde Kit Chaves Jogo Catraca Reversível Soquetes Maleta Promoção promoção</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C74" t="str">
+        <v>https://s.shopee.com.br/3LNHiit93j</v>
+      </c>
+      <c r="D74" t="str">
+        <v>R$ 30,99</v>
+      </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
+      <c r="F74" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>The Perfect Top Insider</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C75" t="str">
+        <v>https://s.shopee.com.br/3B3rWPtmOi</v>
+      </c>
+      <c r="D75" t="str">
+        <v>R$ 135,00</v>
+      </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
+      <c r="F75" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Cortina Blackout PVC Voil Xadrez 1,40 × 1,70 / 2,00 X 1,40</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C76" t="str">
+        <v>https://s.shopee.com.br/30kRK6uPjh</v>
+      </c>
+      <c r="D76" t="str">
+        <v>R$ 36,96</v>
+      </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
+      <c r="F76" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>vestido  midi  de bolso  tamanho  único  g ,veste do 40 só 44, tecido  visco laycra</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Oferta Especial Shopee (0.22)</v>
+      </c>
+      <c r="C77" t="str">
+        <v>https://s.shopee.com.br/2qR17nv34g</v>
+      </c>
+      <c r="D77" t="str">
+        <v>R$ 26,99</v>
+      </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
+      <c r="F77" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Toalha de Mesa Plástico Térmica Impermeável Premium para Mesas 4 CadeiraS / 6 Cadeiras / 8 Cadeiras</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C78" t="str">
+        <v>https://s.shopee.com.br/2g7avUvgPf</v>
+      </c>
+      <c r="D78" t="str">
+        <v>R$ 11,96</v>
+      </c>
+      <c r="E78" t="str">
+        <v/>
+      </c>
+      <c r="F78" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Papel Descartável Air Fryer Antiaderente Para Cozimento 50 Unidades</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C79" t="str">
+        <v>https://s.shopee.com.br/5Aovu5mALA</v>
+      </c>
+      <c r="D79" t="str">
+        <v>R$ 14,39</v>
+      </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
+      <c r="F79" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Prateleira multiuso 4 andares modular.</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Oferta Especial Shopee (0.17)</v>
+      </c>
+      <c r="C80" t="str">
+        <v>https://s.shopee.com.br/50VVhmmng9</v>
+      </c>
+      <c r="D80" t="str">
+        <v>R$ 29,99</v>
+      </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
+      <c r="F80" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Kit Completo p/ Projetor HY320 Mini – Com Suportes e Tampa de Lente - pronto par instalar</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C81" t="str">
+        <v>https://s.shopee.com.br/4qC5VTnR18</v>
+      </c>
+      <c r="D81" t="str">
+        <v>R$ 33,99</v>
+      </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
+      <c r="F81" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Bebedouro Automatico Pet Fonte para Cães e Gatos Silenciosa Bivolt 1,5L</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C82" t="str">
+        <v>https://s.shopee.com.br/4fsfJAo4M7</v>
+      </c>
+      <c r="D82" t="str">
+        <v>R$ 48,99</v>
+      </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
+      <c r="F82" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>QUEIMA DE ESTOQUE Tênis Feminino F1 Branco Casual Barato Do 34 ao 43 Masculino</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C83" t="str">
+        <v>https://s.shopee.com.br/4VZF6rohh6</v>
+      </c>
+      <c r="D83" t="str">
+        <v>R$ 149,90</v>
+      </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
+      <c r="F83" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Kit 5 Cuecas Boxer Sandrini Algodão Adulto Masculinas Elastano Original cueca box Promoção</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C84" t="str">
+        <v>https://s.shopee.com.br/4LFouYpL25</v>
+      </c>
+      <c r="D84" t="str">
+        <v>R$ 24,99</v>
+      </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
+      <c r="F84" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Caixa Caixinha De Som Bluetooth Potente Pendrive Fm Sd Portátil Ipx6</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C85" t="str">
+        <v>https://s.shopee.com.br/4AwOiFpyN4</v>
+      </c>
+      <c r="D85" t="str">
+        <v>R$ 55,00</v>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+      <c r="F85" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Microfone Lapela Sem Fio Duplo Kaidi Profissional Portátil Imã Redondo Anti Ruído Tipo C iPhone Gravação Celular</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Oferta Especial Shopee (0.21)</v>
+      </c>
+      <c r="C86" t="str">
+        <v>https://s.shopee.com.br/40cyVwqbi3</v>
+      </c>
+      <c r="D86" t="str">
+        <v>R$ 74,80</v>
+      </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
+      <c r="F86" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Caixa de Som Grande Amplificada 2000w com Rodinha e 2 Microfones Sem Fio LED MP3</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Oferta Especial Shopee (0.28)</v>
+      </c>
+      <c r="C87" t="str">
+        <v>https://s.shopee.com.br/6VKJUXh5dY</v>
+      </c>
+      <c r="D87" t="str">
+        <v>R$ 531,99</v>
+      </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
+      <c r="F87" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Fone De Ouvido Bluetooth Sem Fio I12 Touch Original Earphone TWS Anatel</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C88" t="str">
+        <v>https://s.shopee.com.br/6L0tIEhiyX</v>
+      </c>
+      <c r="D88" t="str">
+        <v>R$ 45,49</v>
+      </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
+      <c r="F88" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Caixa de Som Portatil Amplificada 2 Altos Falantes Caixinha Grande Potencia Heruz LED Bluetooth Recarregavel</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C89" t="str">
+        <v>https://s.shopee.com.br/6AhT5viMJW</v>
+      </c>
+      <c r="D89" t="str">
+        <v>R$ 163,99</v>
+      </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
+      <c r="F89" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Fone de Ouvido Gamer Com Fio Headset Microfone Controle de Volume Original Inova</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C90" t="str">
+        <v>https://s.shopee.com.br/60O2tcizeV</v>
+      </c>
+      <c r="D90" t="str">
+        <v>R$ 58,90</v>
+      </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
+      <c r="F90" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>CAIXA DE SOM PC GAMER COMPUTADOR KNUP HÓRUS R0850 – MULTIMÍDIA 2.0 | LED COLORIDO | 10W RMS | P2 + USB | WINDOWS / MAC</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C91" t="str">
+        <v>https://s.shopee.com.br/5q4chJjczU</v>
+      </c>
+      <c r="D91" t="str">
+        <v>R$ 74,99</v>
+      </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
+      <c r="F91" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Fone de Ouvido Bluetooth Headphone Sem Fio Inova Original Graves Potentes</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C92" t="str">
+        <v>https://s.shopee.com.br/5flCV0kGKT</v>
+      </c>
+      <c r="D92" t="str">
+        <v>R$ 79,90</v>
+      </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
+      <c r="F92" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Caixinha De Som Caixa Grande Potencia Led Bluetooth 2 Alto Falantes Heruz MP3</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C93" t="str">
+        <v>https://s.shopee.com.br/5VRmIhktfS</v>
+      </c>
+      <c r="D93" t="str">
+        <v>R$ 158,99</v>
+      </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
+      <c r="F93" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Caixa de som Bluetooth Caixinha Grande Com Led RGB Portátil USB 2 Alto Falantes</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C94" t="str">
+        <v>https://s.shopee.com.br/5L8M6OlX0R</v>
+      </c>
+      <c r="D94" t="str">
+        <v>R$ 158,99</v>
+      </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
+      <c r="F94" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Fone de Ouvido - Bluetooth - Sem Fio - Inova - IPhone - Android - Pequeno - Minimalista</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C95" t="str">
+        <v>https://s.shopee.com.br/7pph4zc0vw</v>
+      </c>
+      <c r="D95" t="str">
+        <v>R$ 53,00</v>
+      </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
+      <c r="F95" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Kit 3 Blusas Feminina Cores Brasil Copa Gola Alta Canelada Manga Curta Elegante Confortável</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Oferta Especial Shopee (0.22)</v>
+      </c>
+      <c r="C96" t="str">
+        <v>https://s.shopee.com.br/7fWGsgceGv</v>
+      </c>
+      <c r="D96" t="str">
+        <v>R$ 47,90</v>
+      </c>
+      <c r="E96" t="str">
+        <v/>
+      </c>
+      <c r="F96" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>SAIA FEMININA COURO MIDI ENVELOPE AMARRAÇÃO + MODA SOCIAL</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C97" t="str">
+        <v>https://s.shopee.com.br/7VCqgNdHbu</v>
+      </c>
+      <c r="D97" t="str">
+        <v>R$ 75,58</v>
+      </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
+      <c r="F97" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Blusa Feminina Brasil T-shirt Verão Algodão</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Oferta Especial Shopee (0.28)</v>
+      </c>
+      <c r="C98" t="str">
+        <v>https://s.shopee.com.br/7KtQU4duwt</v>
+      </c>
+      <c r="D98" t="str">
+        <v>R$ 31,96</v>
+      </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
+      <c r="F98" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Conjuntos de manga longa em torno do pescoço impresso moletom e leggings</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C99" t="str">
+        <v>https://s.shopee.com.br/7Aa0HleYHs</v>
+      </c>
+      <c r="D99" t="str">
+        <v>R$ 98,33</v>
+      </c>
+      <c r="E99" t="str">
+        <v/>
+      </c>
+      <c r="F99" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Kit pijama mãe e filha capivara inverno calça estampada malha blusa manga comprida personagens inverno frio longo</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Oferta Especial Shopee (0.21)</v>
+      </c>
+      <c r="C100" t="str">
+        <v>https://s.shopee.com.br/70Ga5SfBcr</v>
+      </c>
+      <c r="D100" t="str">
+        <v>R$ 79,20</v>
+      </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
+      <c r="F100" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Cropped Top Feminino Alcinha Frente Forrada Personalizado Copa 2026 ESTHER BRASIL</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Oferta Especial Shopee (0.2)</v>
+      </c>
+      <c r="C101" t="str">
+        <v>https://s.shopee.com.br/6px9t9foxq</v>
+      </c>
+      <c r="D101" t="str">
+        <v>R$ 29,83</v>
+      </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
+      <c r="F101" t="str">
         <v>Shopee</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F101"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Upload da lista completa do OneDrive
</commit_message>
<xml_diff>
--- a/shopee.xlsx
+++ b/shopee.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F101"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -433,7 +433,7 @@
         <v>R$ 30,99</v>
       </c>
       <c r="E2" t="str">
-        <v>https://m.media-amazon.com/images/I/81MzIgh8luL.jpg</v>
+        <v/>
       </c>
       <c r="F2" t="str">
         <v>Shopee</v>
@@ -441,19 +441,19 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Jogo de Lençol 400 Fios Cama Solteiro Casal Queen King E Berço Micropercal Ponto Palito</v>
+        <v>Kit  Collagen Completo Máscara 500g Shampoo 1L Condicionador 1L Óleo Maca 50ml Tratamento Profissional</v>
       </c>
       <c r="B3" t="str">
-        <v>Oferta Especial Shopee (0.21)</v>
+        <v>Oferta Especial Shopee (0.16)</v>
       </c>
       <c r="C3" t="str">
-        <v>https://s.shopee.com.br/1qYTvxyr5J</v>
+        <v>https://s.shopee.com.br/1gF3jezUQG</v>
       </c>
       <c r="D3" t="str">
-        <v>R$ 27,23</v>
+        <v>R$ 54,00</v>
       </c>
       <c r="E3" t="str">
-        <v>https://down-br.img.susercontent.com/file/br-11134207-7qukw-ljj75v06g0i857</v>
+        <v/>
       </c>
       <c r="F3" t="str">
         <v>Shopee</v>
@@ -461,19 +461,19 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Kit 1 ou 2 Unidades de Veda Porta Ajustável Protetor Rolinho Impermeável 80cm 90cm 100cm</v>
+        <v>Jogo de Lençol 400 Fios Cama Solteiro Casal Queen King E Berço Micropercal Ponto Palito</v>
       </c>
       <c r="B4" t="str">
-        <v>Oferta Especial Shopee (0.24)</v>
+        <v>Oferta Especial Shopee (0.21)</v>
       </c>
       <c r="C4" t="str">
-        <v>https://s.shopee.com.br/1LcDL30l6E</v>
+        <v>https://s.shopee.com.br/1qYTvxyr5J</v>
       </c>
       <c r="D4" t="str">
-        <v>R$ 12,54</v>
+        <v>R$ 27,23</v>
       </c>
       <c r="E4" t="str">
-        <v>https://m.media-amazon.com/images/I/51WhpiChLTL.jpg</v>
+        <v/>
       </c>
       <c r="F4" t="str">
         <v>Shopee</v>
@@ -481,19 +481,19 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Kit Limpador Pastilha de máquina de lavar roupa, comprimido efervescente sólido para remover manchas【】</v>
+        <v>Kit 1 ou 2 Unidades de Veda Porta Ajustável Protetor Rolinho Impermeável 80cm 90cm 100cm</v>
       </c>
       <c r="B5" t="str">
-        <v>Oferta Especial Shopee (0.18)</v>
+        <v>Oferta Especial Shopee (0.24)</v>
       </c>
       <c r="C5" t="str">
-        <v>https://s.shopee.com.br/1VvdXM07lH</v>
+        <v>https://s.shopee.com.br/1LcDL30l6E</v>
       </c>
       <c r="D5" t="str">
-        <v>R$ 859,00</v>
+        <v>R$ 12,54</v>
       </c>
       <c r="E5" t="str">
-        <v>https://m.media-amazon.com/images/I/71MghNSCDPL._AC_UF1000,1000_QL80_.jpg</v>
+        <v/>
       </c>
       <c r="F5" t="str">
         <v>Shopee</v>
@@ -501,19 +501,19 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Kit 3 Peneira Coador De Peneiras Aço Inoxidável Para Cozinha Peneira De Cozinha</v>
+        <v>Kit Limpador Pastilha de máquina de lavar roupa, comprimido efervescente sólido para remover manchas【】</v>
       </c>
       <c r="B6" t="str">
-        <v>Oferta Especial Shopee (0.15)</v>
+        <v>Oferta Especial Shopee (0.18)</v>
       </c>
       <c r="C6" t="str">
-        <v>https://s.shopee.com.br/3g087KrsMi</v>
+        <v>https://s.shopee.com.br/1VvdXM07lH</v>
       </c>
       <c r="D6" t="str">
-        <v>R$ 15,99</v>
+        <v>R$ 859,00</v>
       </c>
       <c r="E6" t="str">
-        <v>https://m.media-amazon.com/images/I/71A3ImQhfHL._AC_UF894,1000_QL80_.jpg</v>
+        <v/>
       </c>
       <c r="F6" t="str">
         <v>Shopee</v>
@@ -521,19 +521,19 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>KIT 1/2/5 Suporte De Parede Multifuncional Caixa De Armazenamento Casa Para Carregar Remoto Um Slot Promoção</v>
+        <v>Kit 3 Peneira Coador De Peneiras Aço Inoxidável Para Cozinha Peneira De Cozinha</v>
       </c>
       <c r="B7" t="str">
-        <v>Oferta Especial Shopee (0.23)</v>
+        <v>Oferta Especial Shopee (0.15)</v>
       </c>
       <c r="C7" t="str">
-        <v>https://s.shopee.com.br/3LNHiit92g</v>
+        <v>https://s.shopee.com.br/3g087KrsMi</v>
       </c>
       <c r="D7" t="str">
-        <v>R$ 959,00</v>
+        <v>R$ 15,99</v>
       </c>
       <c r="E7" t="str">
-        <v>https://down-br.img.susercontent.com/file/br-11134207-7qukw-ljpumel2dxmy85</v>
+        <v/>
       </c>
       <c r="F7" t="str">
         <v>Shopee</v>
@@ -541,19 +541,19 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Mangueira de Jardim Anti-Torção e Anti-Dobras de 5 a 50 Metros</v>
+        <v>Inox Torneira  Prata/Preto Com Chuveiro Com Rotação De 360° Cozinha Luxo Parede Promoção</v>
       </c>
       <c r="B8" t="str">
-        <v>Oferta Especial Shopee (0.21)</v>
+        <v>Oferta Especial Shopee (0.23)</v>
       </c>
       <c r="C8" t="str">
-        <v>https://s.shopee.com.br/3Vghv1sVhj</v>
+        <v>https://s.shopee.com.br/3qJYJdrF1l</v>
       </c>
       <c r="D8" t="str">
-        <v>R$ 17,32</v>
+        <v>R$ 23,99</v>
       </c>
       <c r="E8" t="str">
-        <v>https://down-br.img.susercontent.com/file/br-11134207-7r98o-m4zac7gestxh75</v>
+        <v/>
       </c>
       <c r="F8" t="str">
         <v>Shopee</v>
@@ -561,27 +561,1867 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>KIT 1/2/5 Suporte De Parede Multifuncional Caixa De Armazenamento Casa Para Carregar Remoto Um Slot Promoção</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>https://s.shopee.com.br/3LNHiit92g</v>
+      </c>
+      <c r="D9" t="str">
+        <v>R$ 959,00</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Mangueira de Jardim Anti-Torção e Anti-Dobras de 5 a 50 Metros</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Oferta Especial Shopee (0.21)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>https://s.shopee.com.br/3Vghv1sVhj</v>
+      </c>
+      <c r="D10" t="str">
+        <v>R$ 17,32</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Creme Desodorante Antitranspirante Herbíssimo Care Rosa Mosqueta E Niacinamida Bisnaga 55g</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B11" t="str">
         <v>Oferta Especial Shopee (0.17)</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C11" t="str">
         <v>https://s.shopee.com.br/30kRK6uPie</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D11" t="str">
         <v>R$ 16,99</v>
       </c>
-      <c r="E9" t="str">
-        <v>https://epocacosmeticos.vteximg.com.br/arquivos/ids/792015-800-800/17404927504767.jpg?v=638772260539870000</v>
-      </c>
-      <c r="F9" t="str">
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Kit Maca Power Completo com 7 Produtos – Cronograma Capilar + Máscara 500g, Shampoo 1L, Condicionador 1L  Reparador 50ml</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Oferta Especial Shopee (0.16)</v>
+      </c>
+      <c r="C12" t="str">
+        <v>https://s.shopee.com.br/3B3rWPtmNh</v>
+      </c>
+      <c r="D12" t="str">
+        <v>R$ 78,00</v>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Creme Depilatório Corporal Depilsam Aloe Vera 200G</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Oferta Especial Shopee (0.17)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>https://s.shopee.com.br/2g7avUvgOc</v>
+      </c>
+      <c r="D13" t="str">
+        <v>R$ 24,98</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Protetor de Colchão Impermeável Matelado Varias Cores Para Cama Box Solteiro, Casal, Queen, King, Mini Berço E Berço</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Oferta Especial Shopee (0.24)</v>
+      </c>
+      <c r="C14" t="str">
+        <v>https://s.shopee.com.br/2qR17nv33f</v>
+      </c>
+      <c r="D14" t="str">
+        <v>R$ 15,90</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>KIT 3, 6 e 9 Calcinha Feminina Tanga Infantil Juvenil Algodão Macio Ajuste Perfeito Cores Estampas Sortidas</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C15" t="str">
+        <v>https://s.shopee.com.br/50VVhmmnf6</v>
+      </c>
+      <c r="D15" t="str">
+        <v>R$ 15,90</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>JBSARA Soro Renovador de Retinol 1ml Envio da Coreia 1 peça</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>https://s.shopee.com.br/5Aovu5mAK9</v>
+      </c>
+      <c r="D16" t="str">
+        <v>R$ 349,00</v>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Regata Alça Fina Fitness Blusa Feminino Liso Poliamida Tank Top Slim Camiseta Academia Verão</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>https://s.shopee.com.br/4fsfJAo4L4</v>
+      </c>
+      <c r="D17" t="str">
+        <v>R$ 37,90</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Fórmula de Lyah 60 doses - Suplemento Alimentar</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Oferta Especial Shopee (0.25)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>https://s.shopee.com.br/4qC5VTnR07</v>
+      </c>
+      <c r="D18" t="str">
+        <v>R$ 69,90</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Creme Gel Regenerador Facial Gota de Colágeno Kokeshi 45g</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Oferta Especial Shopee (0.24)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>https://s.shopee.com.br/4LFouYpL12</v>
+      </c>
+      <c r="D19" t="str">
+        <v>R$ 32,83</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Creme Para Pentear Definição Natural 1kg</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>https://s.shopee.com.br/4VZF6rohg5</v>
+      </c>
+      <c r="D20" t="str">
+        <v>R$ 35,75</v>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Cinta Modeladora Espartilho De Emagrecimento-ENVIO IMEDIATO --8888</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Oferta Especial Shopee (0.16)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>https://s.shopee.com.br/40cyVwqbh0</v>
+      </c>
+      <c r="D21" t="str">
+        <v>R$ 22,80</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>1/2/3 Forro Antiderrapante Para Gaveta, Geladeira E Guarda Roupas- Transparente 0,6*3M Evita Deslizamento em Superfícies</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C22" t="str">
+        <v>https://s.shopee.com.br/4AwOiFpyM3</v>
+      </c>
+      <c r="D22" t="str">
+        <v>R$ 23,99</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Kit 10 Marmita conjunto Potes 750ml com Travas Laterais BPA FREE - Alimentos organizadores de congelador</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>https://s.shopee.com.br/6L0tIEhixU</v>
+      </c>
+      <c r="D23" t="str">
+        <v>R$ 21,90</v>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Relógio Masculino digital wr | 100 % qualidade | entrega rápida</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>https://s.shopee.com.br/6VKJUXh5cX</v>
+      </c>
+      <c r="D24" t="str">
+        <v>R$ 12,99</v>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Coberdrom Cobertor Solteiro Casal Queen E King Colcha Dupla Face Edredrom Luxo Pele Carneiro Premium</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>https://s.shopee.com.br/60O2tcizdS</v>
+      </c>
+      <c r="D25" t="str">
+        <v>R$ 94,98</v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Amplificador De Imagem Da Tela Do Celular Lupa 3D 21,6CM*16,6CM*2,7CM Promoção</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>https://s.shopee.com.br/6AhT5viMIV</v>
+      </c>
+      <c r="D26" t="str">
+        <v>R$ 17,99</v>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Óleo de Tratamento SOS Cachos 10 em 1 Multibenefícios 42ml</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>https://s.shopee.com.br/5flCV0kGJQ</v>
+      </c>
+      <c r="D27" t="str">
+        <v>R$ 16,20</v>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Arranjo c/ 3 Trepadeira Folha de HERA + Vaso Trançado Marrom</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Oferta Especial Shopee (0.28)</v>
+      </c>
+      <c r="C28" t="str">
+        <v>https://s.shopee.com.br/5q4chJjcyT</v>
+      </c>
+      <c r="D28" t="str">
+        <v>R$ 16,80</v>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Alvejante Poderoso com Percarbonato de Sódio Tira Manchas Roupas Brancas e Coloridas -GF Agro</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Oferta Especial Shopee (0.22)</v>
+      </c>
+      <c r="C29" t="str">
+        <v>https://s.shopee.com.br/5L8M6OlWzO</v>
+      </c>
+      <c r="D29" t="str">
+        <v>R$ 11,99</v>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>30 unidades cabide redondo resistente adulto</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Oferta Especial Shopee (0.17)</v>
+      </c>
+      <c r="C30" t="str">
+        <v>https://s.shopee.com.br/5VRmIhkteR</v>
+      </c>
+      <c r="D30" t="str">
+        <v>R$ 19,98</v>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Principia Kit Completo Peles Sensíveis c/ Gel de Limpeza Gl-02 + Creme Hidratante CH-01 + Protetor Solar PS-01 FPS 60</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C31" t="str">
+        <v>https://s.shopee.com.br/7fWGsgceFs</v>
+      </c>
+      <c r="D31" t="str">
+        <v>R$ 116,25</v>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+      <c r="F31" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Cera Espelhamento RENOVE – Remove Riscos Superficiais, Repele Água, Proteção Sol, Brilho Intenso</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Oferta Especial Shopee (0.24)</v>
+      </c>
+      <c r="C32" t="str">
+        <v>https://s.shopee.com.br/7pph4zc0uv</v>
+      </c>
+      <c r="D32" t="str">
+        <v>R$ 17,99</v>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Kit 10, 5 Cueca Masculina Box Adulto Microfibra Forro 100% Algodão Cores Variadas</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C33" t="str">
+        <v>https://s.shopee.com.br/7KtQU4duvq</v>
+      </c>
+      <c r="D33" t="str">
+        <v>R$ 26,80</v>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Mini Umidificador Difusor Aromatizador Egg Portátil Usb Led Aromatizador De Ambiente Purificador De Ar Casa Escritório</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C34" t="str">
+        <v>https://s.shopee.com.br/7VCqgNdHat</v>
+      </c>
+      <c r="D34" t="str">
+        <v>R$ 16,99</v>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Luminária Despertador Com Luz Led Bluetooth Caixa  Som Relógio Digital  Carregamento Indução Abajur</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C35" t="str">
+        <v>https://s.shopee.com.br/70Ga5SfBbo</v>
+      </c>
+      <c r="D35" t="str">
+        <v>R$ 34,90</v>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>kit Coala Home Chá Branco</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C36" t="str">
+        <v>https://s.shopee.com.br/7Aa0HleYGr</v>
+      </c>
+      <c r="D36" t="str">
+        <v>R$ 69,99</v>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Cafe Graos Torra Media Gourmet Café Italle 1kg</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Oferta Especial Shopee (0.28)</v>
+      </c>
+      <c r="C37" t="str">
+        <v>https://s.shopee.com.br/6fdjgqgSHm</v>
+      </c>
+      <c r="D37" t="str">
+        <v>R$ 71,30</v>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Cinto Masculino Feminino Tecido Trançado Elástico Fivela De Metal</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Oferta Especial Shopee (0.17)</v>
+      </c>
+      <c r="C38" t="str">
+        <v>https://s.shopee.com.br/6px9t9fowp</v>
+      </c>
+      <c r="D38" t="str">
+        <v>R$ 10,99</v>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Kit de 72 unidades de Xuxinha de cabelo elastico de para cabelo feminino rabicó</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C39" t="str">
+        <v>https://s.shopee.com.br/901eT8XZYG</v>
+      </c>
+      <c r="D39" t="str">
+        <v>R$ 10,87</v>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Manta Cobertor Microfibra Casal Queen King Quentinha Antialérgico Poá Habitat</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Oferta Especial Shopee (0.21)</v>
+      </c>
+      <c r="C40" t="str">
+        <v>https://s.shopee.com.br/9AL4fRWwDJ</v>
+      </c>
+      <c r="D40" t="str">
+        <v>R$ 52,89</v>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Pistola Elétrica Para Pintura Pulverizador de Tinta com Bico de Metal e Compressor 450w - TSSAPER</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C41" t="str">
+        <v>https://s.shopee.com.br/8fOo4WYqEE</v>
+      </c>
+      <c r="D41" t="str">
+        <v>R$ 137,45</v>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Lençol Com Elástico Premium Avulso 400 Fios Percal Liso Toque Macio Acetinado</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C42" t="str">
+        <v>https://s.shopee.com.br/8piEGpYCtH</v>
+      </c>
+      <c r="D42" t="str">
+        <v>R$ 18,80</v>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Balança Corporal Transparente Quadrada Digital Até 180kg Com Vidro Temperado Premium</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C43" t="str">
+        <v>https://s.shopee.com.br/8Klxfua6uC</v>
+      </c>
+      <c r="D43" t="str">
+        <v>R$ 32,99</v>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>2025 Nova Série 8 Relógio T800 Ultra Smart Watch Esportivo Sem Fio À Prova D'água T800 Ultra2 MAX</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Oferta Especial Shopee (0.16)</v>
+      </c>
+      <c r="C44" t="str">
+        <v>https://s.shopee.com.br/8V5NsDZTZF</v>
+      </c>
+      <c r="D44" t="str">
+        <v>R$ 38,99</v>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Protetor Solar Facial PS-01 FPS 60 Principia</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C45" t="str">
+        <v>https://s.shopee.com.br/8097HIbNaA</v>
+      </c>
+      <c r="D45" t="str">
+        <v>R$ 49,00</v>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+      <c r="F45" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Leggings canelada de cintura larga e cor sólida para atividades esportivas.</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C46" t="str">
+        <v>https://s.shopee.com.br/8ASXTbakFD</v>
+      </c>
+      <c r="D46" t="str">
+        <v>R$ 29,99</v>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Blusa Feminina Manga 3/4 Novas Cores Tecido Crepe Moda Evangelica Detalhe Social Elegante</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Oferta Especial Shopee (0.34)</v>
+      </c>
+      <c r="C47" t="str">
+        <v>https://s.shopee.com.br/AKX23aSUqe</v>
+      </c>
+      <c r="D47" t="str">
+        <v>R$ 26,99</v>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Fita Multiuso Manta Asfaltica Adesiva para Reparos Rufo Calha Telhado Veda Tudo 10cm 20cm 30cm POR METRO</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Oferta Especial Shopee (0.16)</v>
+      </c>
+      <c r="C48" t="str">
+        <v>https://s.shopee.com.br/AUqSFtRrVh</v>
+      </c>
+      <c r="D48" t="str">
+        <v>R$ 999,00</v>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Blusa Manga 3/4 Detalhe Em V Novas Cores Verão Tendência Moda Feminina</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Oferta Especial Shopee (0.17)</v>
+      </c>
+      <c r="C49" t="str">
+        <v>https://s.shopee.com.br/9zuBeyTlWc</v>
+      </c>
+      <c r="D49" t="str">
+        <v>R$ 26,99</v>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Kit M10 Bluetooth 5.3 Sem Fio TWS Fones De Ouvido Estéreo Com Carregador Power Bank Atualizado 100 % Novo Alto-Falante</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C50" t="str">
+        <v>https://s.shopee.com.br/AADbrHT8Bf</v>
+      </c>
+      <c r="D50" t="str">
+        <v>R$ 25,89</v>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Shampoo Tonalizante Escurecedor S/ Amônia Avelã, Marsala, Loiro, Vermelho Ruivo 100% Natural Matizze</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C51" t="str">
+        <v>https://s.shopee.com.br/9fHLGMV2Ca</v>
+      </c>
+      <c r="D51" t="str">
+        <v>R$ 17,89</v>
+      </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
+      <c r="F51" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Kit de Óleo Capilar - Cronograma Terapia Capilar - 100% natural - 60ml</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Oferta Especial Shopee (0.2)</v>
+      </c>
+      <c r="C52" t="str">
+        <v>https://s.shopee.com.br/9palSfUOrd</v>
+      </c>
+      <c r="D52" t="str">
+        <v>R$ 15,30</v>
+      </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
+      <c r="F52" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Carregador Portátil Mini Power Bank 10000mAh Com 02 Saídas Tipo-C / Lightning</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Oferta Especial Shopee (0.34)</v>
+      </c>
+      <c r="C53" t="str">
+        <v>https://s.shopee.com.br/9KeUrkWIsY</v>
+      </c>
+      <c r="D53" t="str">
+        <v>R$ 32,99</v>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+      <c r="F53" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Mini Barbeador Elétrico Portátil À Prova D'água De Dupla Finalidade Tipo c De Carga Rápida Aparador De Barba De Bolso</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C54" t="str">
+        <v>https://s.shopee.com.br/9Uxv43VfXb</v>
+      </c>
+      <c r="D54" t="str">
+        <v>R$ 16,99</v>
+      </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
+      <c r="F54" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Trava Óculos Antiderrapante Silicone Kit Não Cai Do Rosto Gancho Orelha Haste Conforto</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C55" t="str">
+        <v>https://s.shopee.com.br/1BIn8k1OS0</v>
+      </c>
+      <c r="D55" t="str">
+        <v>R$ 700,00</v>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Kit 3 Bermudas Masculina Esportivo Academia Praia Com  Bolsos E Refletivo</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C56" t="str">
+        <v>https://s.shopee.com.br/10zMwR21mz</v>
+      </c>
+      <c r="D56" t="str">
+        <v>R$ 44,04</v>
+      </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+      <c r="F56" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Kit Com 10 ou 4 Cuecas Boxers Premium Masculina Adulto de Microfibra</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C57" t="str">
+        <v>https://s.shopee.com.br/qfwk82f7y</v>
+      </c>
+      <c r="D57" t="str">
+        <v>R$ 24,98</v>
+      </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
+      <c r="F57" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Shorts modeladores sem costura com forro de microfibra</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Oferta Especial Shopee (0.16)</v>
+      </c>
+      <c r="C58" t="str">
+        <v>https://s.shopee.com.br/gMWXp3ISx</v>
+      </c>
+      <c r="D58" t="str">
+        <v>R$ 19,24</v>
+      </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
+      <c r="F58" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Kit 4pçs Toalhas de Banho 140x70cm 100% Algodão Premium Coleção Difiori</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C59" t="str">
+        <v>https://s.shopee.com.br/W36LW3vnw</v>
+      </c>
+      <c r="D59" t="str">
+        <v>R$ 69,99</v>
+      </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
+      <c r="F59" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Protetor para Colchão Lençol Impermeável Matelado Com Toque Silencioso</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Oferta Especial Shopee (0.2)</v>
+      </c>
+      <c r="C60" t="str">
+        <v>https://s.shopee.com.br/Ljg9D4Z8v</v>
+      </c>
+      <c r="D60" t="str">
+        <v>R$ 14,90</v>
+      </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
+      <c r="F60" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Carregador Portátil Mini Power Bank 10000mAh Com 02 Saídas Tipo-C / Lightning</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Oferta Especial Shopee (0.34)</v>
+      </c>
+      <c r="C61" t="str">
+        <v>https://s.shopee.com.br/BQFwu5CTu</v>
+      </c>
+      <c r="D61" t="str">
+        <v>R$ 31,99</v>
+      </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
+      <c r="F61" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Gel Dental Pro White Hinode 90g</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Oferta Especial Shopee (0.28)</v>
+      </c>
+      <c r="C62" t="str">
+        <v>https://s.shopee.com.br/16pkb5pot</v>
+      </c>
+      <c r="D62" t="str">
+        <v>R$ 16,90</v>
+      </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
+      <c r="F62" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2 Pcs Meias De Silicone Para O Cuidado Dos Pés Gel Hidratante Anti-Rachaduras Removedor De Pele Morta</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C63" t="str">
+        <v>https://s.shopee.com.br/2VoAjBwJkO</v>
+      </c>
+      <c r="D63" t="str">
+        <v>R$ 999,00</v>
+      </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
+      <c r="F63" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Ventilador de Mesa 40 cm 10 Pás com 3 Velocidades Ventisol Turbo 10</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Oferta Especial Shopee (0.48)</v>
+      </c>
+      <c r="C64" t="str">
+        <v>https://s.shopee.com.br/2LUkWswx5N</v>
+      </c>
+      <c r="D64" t="str">
+        <v>R$ 149,90</v>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+      <c r="F64" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Extensão cabo PP Eletrica 50 Metros Reforçada Profissional 10/20a</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C65" t="str">
+        <v>https://s.shopee.com.br/2BBKKZxaQM</v>
+      </c>
+      <c r="D65" t="str">
+        <v>R$ 49,00</v>
+      </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
+      <c r="F65" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Copo Garrafa Térmica Grande Em Aço Inox Com Alça E Canudo Metal 1200ML</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Oferta Especial Shopee (0.34)</v>
+      </c>
+      <c r="C66" t="str">
+        <v>https://s.shopee.com.br/20ru8GyDlL</v>
+      </c>
+      <c r="D66" t="str">
+        <v>R$ 36,99</v>
+      </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
+      <c r="F66" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Cueiro Estampado Flanelado Bebê Kit 3 Unidades 80X50CM Papi/Incomfral</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C67" t="str">
+        <v>https://s.shopee.com.br/1qYTvxyr6K</v>
+      </c>
+      <c r="D67" t="str">
+        <v>R$ 19,99</v>
+      </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
+      <c r="F67" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Garrafa Inox Térmica Com Capinha Protetora De Silicone Antiderrapante 1000ML</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Oferta Especial Shopee (0.34)</v>
+      </c>
+      <c r="C68" t="str">
+        <v>https://s.shopee.com.br/1gF3jezURJ</v>
+      </c>
+      <c r="D68" t="str">
+        <v>R$ 33,99</v>
+      </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
+      <c r="F68" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>5/10/15/20 Metros Adesivo Papel de Parede Autocolante 5m x 45cm Madeira Mármore Geométrico 2,25m² Y2</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C69" t="str">
+        <v>https://s.shopee.com.br/1VvdXM07mI</v>
+      </c>
+      <c r="D69" t="str">
+        <v>R$ 13,99</v>
+      </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
+      <c r="F69" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Cesto Pão Porta Pães Bolacha Biscoito Organizador MDF Retrátil Cozinha Armazenamento</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C70" t="str">
+        <v>https://s.shopee.com.br/1LcDL30l7H</v>
+      </c>
+      <c r="D70" t="str">
+        <v>R$ 28,00</v>
+      </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
+      <c r="F70" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>46 Peças Verde Kit Chaves Jogo Catraca Reversível Soquetes Maleta Promoção</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C71" t="str">
+        <v>https://s.shopee.com.br/3qJYJdrF2m</v>
+      </c>
+      <c r="D71" t="str">
+        <v>R$ 30,99</v>
+      </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
+      <c r="F71" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Kit Espátula Desencravador Slim Podologia - 3 Peças N206, N214 e Formão N254</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C72" t="str">
+        <v>https://s.shopee.com.br/3g087KrsNl</v>
+      </c>
+      <c r="D72" t="str">
+        <v>R$ 13,99</v>
+      </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
+      <c r="F72" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Kit 5 Toalha de Banho Maldivas 100% algodão 60x120cm Sortidas</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Oferta Especial Shopee (0.25)</v>
+      </c>
+      <c r="C73" t="str">
+        <v>https://s.shopee.com.br/3Vghv1sVik</v>
+      </c>
+      <c r="D73" t="str">
+        <v>R$ 54,45</v>
+      </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
+      <c r="F73" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>40/46 Peças Verde Kit Chaves Jogo Catraca Reversível Soquetes Maleta Promoção promoção</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C74" t="str">
+        <v>https://s.shopee.com.br/3LNHiit93j</v>
+      </c>
+      <c r="D74" t="str">
+        <v>R$ 30,99</v>
+      </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
+      <c r="F74" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>The Perfect Top Insider</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C75" t="str">
+        <v>https://s.shopee.com.br/3B3rWPtmOi</v>
+      </c>
+      <c r="D75" t="str">
+        <v>R$ 135,00</v>
+      </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
+      <c r="F75" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Cortina Blackout PVC Voil Xadrez 1,40 × 1,70 / 2,00 X 1,40</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C76" t="str">
+        <v>https://s.shopee.com.br/30kRK6uPjh</v>
+      </c>
+      <c r="D76" t="str">
+        <v>R$ 36,96</v>
+      </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
+      <c r="F76" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>vestido  midi  de bolso  tamanho  único  g ,veste do 40 só 44, tecido  visco laycra</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Oferta Especial Shopee (0.22)</v>
+      </c>
+      <c r="C77" t="str">
+        <v>https://s.shopee.com.br/2qR17nv34g</v>
+      </c>
+      <c r="D77" t="str">
+        <v>R$ 26,99</v>
+      </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
+      <c r="F77" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Toalha de Mesa Plástico Térmica Impermeável Premium para Mesas 4 CadeiraS / 6 Cadeiras / 8 Cadeiras</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C78" t="str">
+        <v>https://s.shopee.com.br/2g7avUvgPf</v>
+      </c>
+      <c r="D78" t="str">
+        <v>R$ 11,96</v>
+      </c>
+      <c r="E78" t="str">
+        <v/>
+      </c>
+      <c r="F78" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Papel Descartável Air Fryer Antiaderente Para Cozimento 50 Unidades</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C79" t="str">
+        <v>https://s.shopee.com.br/5Aovu5mALA</v>
+      </c>
+      <c r="D79" t="str">
+        <v>R$ 14,39</v>
+      </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
+      <c r="F79" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Prateleira multiuso 4 andares modular.</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Oferta Especial Shopee (0.17)</v>
+      </c>
+      <c r="C80" t="str">
+        <v>https://s.shopee.com.br/50VVhmmng9</v>
+      </c>
+      <c r="D80" t="str">
+        <v>R$ 29,99</v>
+      </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
+      <c r="F80" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Kit Completo p/ Projetor HY320 Mini – Com Suportes e Tampa de Lente - pronto par instalar</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Oferta Especial Shopee (0.15)</v>
+      </c>
+      <c r="C81" t="str">
+        <v>https://s.shopee.com.br/4qC5VTnR18</v>
+      </c>
+      <c r="D81" t="str">
+        <v>R$ 33,99</v>
+      </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
+      <c r="F81" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Bebedouro Automatico Pet Fonte para Cães e Gatos Silenciosa Bivolt 1,5L</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C82" t="str">
+        <v>https://s.shopee.com.br/4fsfJAo4M7</v>
+      </c>
+      <c r="D82" t="str">
+        <v>R$ 48,99</v>
+      </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
+      <c r="F82" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>QUEIMA DE ESTOQUE Tênis Feminino F1 Branco Casual Barato Do 34 ao 43 Masculino</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C83" t="str">
+        <v>https://s.shopee.com.br/4VZF6rohh6</v>
+      </c>
+      <c r="D83" t="str">
+        <v>R$ 149,90</v>
+      </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
+      <c r="F83" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Kit 5 Cuecas Boxer Sandrini Algodão Adulto Masculinas Elastano Original cueca box Promoção</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Oferta Especial Shopee (0.19)</v>
+      </c>
+      <c r="C84" t="str">
+        <v>https://s.shopee.com.br/4LFouYpL25</v>
+      </c>
+      <c r="D84" t="str">
+        <v>R$ 24,99</v>
+      </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
+      <c r="F84" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Caixa Caixinha De Som Bluetooth Potente Pendrive Fm Sd Portátil Ipx6</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C85" t="str">
+        <v>https://s.shopee.com.br/4AwOiFpyN4</v>
+      </c>
+      <c r="D85" t="str">
+        <v>R$ 55,00</v>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+      <c r="F85" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Microfone Lapela Sem Fio Duplo Kaidi Profissional Portátil Imã Redondo Anti Ruído Tipo C iPhone Gravação Celular</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Oferta Especial Shopee (0.21)</v>
+      </c>
+      <c r="C86" t="str">
+        <v>https://s.shopee.com.br/40cyVwqbi3</v>
+      </c>
+      <c r="D86" t="str">
+        <v>R$ 74,80</v>
+      </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
+      <c r="F86" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Caixa de Som Grande Amplificada 2000w com Rodinha e 2 Microfones Sem Fio LED MP3</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Oferta Especial Shopee (0.28)</v>
+      </c>
+      <c r="C87" t="str">
+        <v>https://s.shopee.com.br/6VKJUXh5dY</v>
+      </c>
+      <c r="D87" t="str">
+        <v>R$ 531,99</v>
+      </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
+      <c r="F87" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Fone De Ouvido Bluetooth Sem Fio I12 Touch Original Earphone TWS Anatel</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C88" t="str">
+        <v>https://s.shopee.com.br/6L0tIEhiyX</v>
+      </c>
+      <c r="D88" t="str">
+        <v>R$ 45,49</v>
+      </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
+      <c r="F88" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Caixa de Som Portatil Amplificada 2 Altos Falantes Caixinha Grande Potencia Heruz LED Bluetooth Recarregavel</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C89" t="str">
+        <v>https://s.shopee.com.br/6AhT5viMJW</v>
+      </c>
+      <c r="D89" t="str">
+        <v>R$ 163,99</v>
+      </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
+      <c r="F89" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Fone de Ouvido Gamer Com Fio Headset Microfone Controle de Volume Original Inova</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C90" t="str">
+        <v>https://s.shopee.com.br/60O2tcizeV</v>
+      </c>
+      <c r="D90" t="str">
+        <v>R$ 58,90</v>
+      </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
+      <c r="F90" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>CAIXA DE SOM PC GAMER COMPUTADOR KNUP HÓRUS R0850 – MULTIMÍDIA 2.0 | LED COLORIDO | 10W RMS | P2 + USB | WINDOWS / MAC</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C91" t="str">
+        <v>https://s.shopee.com.br/5q4chJjczU</v>
+      </c>
+      <c r="D91" t="str">
+        <v>R$ 74,99</v>
+      </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
+      <c r="F91" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Fone de Ouvido Bluetooth Headphone Sem Fio Inova Original Graves Potentes</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Oferta Especial Shopee (0.23)</v>
+      </c>
+      <c r="C92" t="str">
+        <v>https://s.shopee.com.br/5flCV0kGKT</v>
+      </c>
+      <c r="D92" t="str">
+        <v>R$ 79,90</v>
+      </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
+      <c r="F92" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Caixinha De Som Caixa Grande Potencia Led Bluetooth 2 Alto Falantes Heruz MP3</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C93" t="str">
+        <v>https://s.shopee.com.br/5VRmIhktfS</v>
+      </c>
+      <c r="D93" t="str">
+        <v>R$ 158,99</v>
+      </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
+      <c r="F93" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Caixa de som Bluetooth Caixinha Grande Com Led RGB Portátil USB 2 Alto Falantes</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Oferta Especial Shopee (0.33)</v>
+      </c>
+      <c r="C94" t="str">
+        <v>https://s.shopee.com.br/5L8M6OlX0R</v>
+      </c>
+      <c r="D94" t="str">
+        <v>R$ 158,99</v>
+      </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
+      <c r="F94" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Fone de Ouvido - Bluetooth - Sem Fio - Inova - IPhone - Android - Pequeno - Minimalista</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C95" t="str">
+        <v>https://s.shopee.com.br/7pph4zc0vw</v>
+      </c>
+      <c r="D95" t="str">
+        <v>R$ 53,00</v>
+      </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
+      <c r="F95" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Kit 3 Blusas Feminina Cores Brasil Copa Gola Alta Canelada Manga Curta Elegante Confortável</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Oferta Especial Shopee (0.22)</v>
+      </c>
+      <c r="C96" t="str">
+        <v>https://s.shopee.com.br/7fWGsgceGv</v>
+      </c>
+      <c r="D96" t="str">
+        <v>R$ 47,90</v>
+      </c>
+      <c r="E96" t="str">
+        <v/>
+      </c>
+      <c r="F96" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>SAIA FEMININA COURO MIDI ENVELOPE AMARRAÇÃO + MODA SOCIAL</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C97" t="str">
+        <v>https://s.shopee.com.br/7VCqgNdHbu</v>
+      </c>
+      <c r="D97" t="str">
+        <v>R$ 75,58</v>
+      </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
+      <c r="F97" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Blusa Feminina Brasil T-shirt Verão Algodão</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Oferta Especial Shopee (0.28)</v>
+      </c>
+      <c r="C98" t="str">
+        <v>https://s.shopee.com.br/7KtQU4duwt</v>
+      </c>
+      <c r="D98" t="str">
+        <v>R$ 31,96</v>
+      </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
+      <c r="F98" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Conjuntos de manga longa em torno do pescoço impresso moletom e leggings</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Oferta Especial Shopee (0.18)</v>
+      </c>
+      <c r="C99" t="str">
+        <v>https://s.shopee.com.br/7Aa0HleYHs</v>
+      </c>
+      <c r="D99" t="str">
+        <v>R$ 98,33</v>
+      </c>
+      <c r="E99" t="str">
+        <v/>
+      </c>
+      <c r="F99" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Kit pijama mãe e filha capivara inverno calça estampada malha blusa manga comprida personagens inverno frio longo</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Oferta Especial Shopee (0.21)</v>
+      </c>
+      <c r="C100" t="str">
+        <v>https://s.shopee.com.br/70Ga5SfBcr</v>
+      </c>
+      <c r="D100" t="str">
+        <v>R$ 79,20</v>
+      </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
+      <c r="F100" t="str">
+        <v>Shopee</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Cropped Top Feminino Alcinha Frente Forrada Personalizado Copa 2026 ESTHER BRASIL</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Oferta Especial Shopee (0.2)</v>
+      </c>
+      <c r="C101" t="str">
+        <v>https://s.shopee.com.br/6px9t9foxq</v>
+      </c>
+      <c r="D101" t="str">
+        <v>R$ 29,83</v>
+      </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
+      <c r="F101" t="str">
         <v>Shopee</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F101"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Correcao critica na formatacao de precos da Shopee
</commit_message>
<xml_diff>
--- a/shopee.xlsx
+++ b/shopee.xlsx
@@ -510,7 +510,7 @@
         <v>https://s.shopee.com.br/1VvdXM07lH</v>
       </c>
       <c r="D6" t="str">
-        <v>R$ 859,00</v>
+        <v>R$ 8,59</v>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -570,7 +570,7 @@
         <v>https://s.shopee.com.br/3LNHiit92g</v>
       </c>
       <c r="D9" t="str">
-        <v>R$ 959,00</v>
+        <v>R$ 9,59</v>
       </c>
       <c r="E9" t="str">
         <v/>
@@ -710,7 +710,7 @@
         <v>https://s.shopee.com.br/5Aovu5mAK9</v>
       </c>
       <c r="D16" t="str">
-        <v>R$ 349,00</v>
+        <v>R$ 3,49</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -1350,7 +1350,7 @@
         <v>https://s.shopee.com.br/AUqSFtRrVh</v>
       </c>
       <c r="D48" t="str">
-        <v>R$ 999,00</v>
+        <v>R$ 9,99</v>
       </c>
       <c r="E48" t="str">
         <v/>
@@ -1490,7 +1490,7 @@
         <v>https://s.shopee.com.br/1BIn8k1OS0</v>
       </c>
       <c r="D55" t="str">
-        <v>R$ 700,00</v>
+        <v>R$ 7,00</v>
       </c>
       <c r="E55" t="str">
         <v/>
@@ -1650,7 +1650,7 @@
         <v>https://s.shopee.com.br/2VoAjBwJkO</v>
       </c>
       <c r="D63" t="str">
-        <v>R$ 999,00</v>
+        <v>R$ 9,99</v>
       </c>
       <c r="E63" t="str">
         <v/>

</xml_diff>

<commit_message>
Upload de 30 produtos do Mercado Livre com imagens reais extraídas com sucesso
</commit_message>
<xml_diff>
--- a/shopee.xlsx
+++ b/shopee.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F131"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2419,9 +2419,609 @@
         <v>Shopee</v>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>Massageador Pistola Elétrica Profissional Muscular Portátil Aparelho Fisioterapia Corporal, 6 Velocidades 4 Cabeças De Massagem - Micgeek 127/220v Variado</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C102" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BIdR1WaJ53Tvir3NVrAy9ELSCXHbgNOc0sAJhdOgm%2FUX0l8AmzOMvn%2BsPUQ4uymir3ZOxC5QPTnDlIFhP4vzw2WLe%2BsoSt17TpFgEcf3Bhr3cdHQu7IKbxxKIWLHtmHH6P%2Bjq6UDkF7UvS0Wz%2BFRJ7OnQwdwePb5%2BWZxE4XGDwaXeL%2Bk7J5eQWpPfQmu96MaWiwbrA%3D%3D</v>
+      </c>
+      <c r="D102" t="str">
+        <v>R$ 68,12</v>
+      </c>
+      <c r="E102" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_860621-MLA98512896914_112025-O.webp</v>
+      </c>
+      <c r="F102" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Nebulizador Inalador Portátil Marca Bahrein Sem Fio A Pilha Ou Cabo Usb Cor Branco Com Azul Compacto Mesh Bivolt Nebulizador Com Rede Vibratória Aparelho Para Inalação Inalador Silencioso 127/220v</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C103" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BLUsfYGxmz6NeXmI%2FIcQPf8LbaT%2FnRpATLGwv%2BPsK4XuOvwfY0yXWovBvsf4rfYuffTOyI4974%2F2aoJaxODiEjN5MtZo1%2FVM4CQfCLvJq8hQEmNHIc5rknyihT1ueQEq%2FbvSBg3cshuWdBRSBvbUD%2Fbx2%2Fd0gQWrr7UmvXdkOJqtoZRq%2BZZML6ySoqczEirKzpjtVQ%3D%3D</v>
+      </c>
+      <c r="D103" t="str">
+        <v>R$ 58,65</v>
+      </c>
+      <c r="E103" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_698758-MLA99675445992_122025-O.webp</v>
+      </c>
+      <c r="F103" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Jaqueta De Couro Masculino Slim Inverno Frio Sem Capuz Preto G Liso</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C104" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BP646zFHJrZUEXwmDgrU9F5%2BSt9Xb7nlbIYaCLr7VR3oOVF5eBsd4hZIJat4k5%2BKItwR%2BEJdv10ngdZVx4o%2B0Nv3341XFkvws9vtueRfVqDXHs%2FQ4zR0Uiat%2FOr7m%2Fse8gmK0dq3eMXUghJ43hDmFp5zJ86X3oYVr%2FucZMV%2Bv4Y0FkOYYyhNHfrIa%2F7QnLMSDWW0xA%3D%3D</v>
+      </c>
+      <c r="D104" t="str">
+        <v>R$ 128,97</v>
+      </c>
+      <c r="E104" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_947582-MLB108560307405_032026-O.webp</v>
+      </c>
+      <c r="F104" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>Barbeador E Cortador De Cabelo 3 Em 1 Kemei Km-6558 Preto 127/220v</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C105" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BKGAc8NVrrTQ8Xahm3yLp33BP0h1LMtTp0kz7lk0JOrYSytzGk6NUxmpQM9u7qjoIGEjWZZ%2F8kzaiWTRi9jmr3OXlxsczHY%2FeijNImUkeq93C0iyiOABz%2BMfavLhPxOi%2BF9m0u31X6tInaNOVkdtvqdbPK%2F1qkw9UX4F9tABNJf37IVk%2BJbVeHPbDYioZxhzm4Brmg%3D%3D</v>
+      </c>
+      <c r="D105" t="str">
+        <v>R$ 139,90</v>
+      </c>
+      <c r="E105" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_638009-MLU77163689638_072024-O.webp</v>
+      </c>
+      <c r="F105" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Gel Lubrificante Íntimo 2 Em 1 K-med Frasco 203g</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C106" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BDYI10h2kHVVJkz4AO87GEBYwRLDI%2BygkWI%2Bs0fJCVJCDU6Hqghg2nhpjKesI1nxcBTX7QDRHQpgMgGBng3DpM93gejpLqZ18YOXUUtqRN0g4MCGIv76QMpk%2Fu8YtkGRaPPC%2BO4xgC%2Fbt4FS%2FXRCOBRbs%2BQz5PGWWuMxb2AdzFi1%2FxC6RI%2FjEhhwi1KXxCFOvrVFrw%3D%3D</v>
+      </c>
+      <c r="D106" t="str">
+        <v>R$ 21,37</v>
+      </c>
+      <c r="E106" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_743442-MLA74072235764_012024-O.webp</v>
+      </c>
+      <c r="F106" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Perfume Hugo Boss Reversed Edt 75ml</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C107" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BOluylHKVOtVjbexLhOqIhLUZcwu7oMhP01Wr7Pf6VCrddTawB15vup6lOD60LRwAy6aYuFaMawl%2BEwEwNYW0qIwledXyg%2BK%2BT7JK9HKD%2BPY1sFWxgECf7i%2BmXKuvyKj4QkuwsDYwYKh%2FUcH25ZIUUpAiJNHip2FBja7OceF7VypwkSfCstrKZdh19mbnVvakQjEzSw%3D</v>
+      </c>
+      <c r="D107" t="str">
+        <v>R$ 639,29</v>
+      </c>
+      <c r="E107" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_976037-MLU73883770497_012024-O.webp</v>
+      </c>
+      <c r="F107" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Torneira Dazie Metais Com Filtro Cozinha Para Parede Flexível Móvel Em Abs Cromado Filtro Carbon Block Purificador De Agua Com 2 Velas Extras Brilhante</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C108" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BFmmlq8Ck1kmKMSiDK3vdTHSb7bauCF82haCxWF4P%2FnFbKfzZUJ5xSCIaGFJrobqioUXbHu3zmjhZ%2BvNqdSE5gD3DlkMexcHYqI%2Fnn65CDVg6Y4Yf%2BdqyZ556xHzfO9qPUS1vnOsuraCLn7Z2msvgIj2TdThybJ5XCoX7KFlYIWWHfGFqzaUig1U1FotuDvRZ7xtvw%3D%3D</v>
+      </c>
+      <c r="D108" t="str">
+        <v>R$ 119,99</v>
+      </c>
+      <c r="E108" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_840765-MLA100039591131_122025-O.webp</v>
+      </c>
+      <c r="F108" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Creme Multirreparador Calmante Cicaplast Baume B5+ Para Todos Os Tipos De Pele Com 40ml La Roche Posay Todo Tipo De Pele Dia/noite</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C109" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BI%2FcBdhYbiDvde3Mg3U38pUiA49SCf%2B8oh57lVT4d8NimkkpitTZWHfQBYRbrhZXb%2FsfwbuFhW9vtEhq2JnbvZFstRKVev%2FJXJVSxeeFYZcsxzBl0yN6I4N92Hz6v9yyY42Wih9o9R0hE3kRvO5C0%2B1Km5TShkrZutiZ4auQbEEPqHEBxRolXOkpsiELlF9nxelsM3s%3D</v>
+      </c>
+      <c r="D109" t="str">
+        <v>R$ 106,90</v>
+      </c>
+      <c r="E109" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_653286-MLA88348742037_072025-O.webp</v>
+      </c>
+      <c r="F109" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>Creatina Monohidratada 250g Growth Supplements - Sem Sabor Em Pó</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C110" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BB%2BsgDjQbnSHDZ5Vs76Smt08qiRMNRgvSXc6G%2F2EjesZZlsfIYOHJ%2BfY%2BF%2BwUMbiG709QTPE5dJvGw4CXWQeGWGeMNQe3pLb%2BvoRTID7rIQ2mEtMVy2vDJ92f40B7eJxfbjN1%2FZ3bOm6JFQPSey1WkJRDsGs3yZP%2FaZEfIH2zWBWqWwCA%2BC%2BpJFr5UWaIpjGiTGAOqc%3D</v>
+      </c>
+      <c r="D110" t="str">
+        <v>R$ 64,90</v>
+      </c>
+      <c r="E110" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_662415-MLA97812910758_112025-O.webp</v>
+      </c>
+      <c r="F110" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>Kit 4 Camiseta Dry-fit Sandrini Masculina Academia Caminhada</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C111" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BPiGFOQo7PFZvEC7vM6sm9mBwvXyom%2BM%2FJW%2BsYRMHq5JE2u5NT%2B0TIMuZAS5dVo2TvzqLgq3QbTYHKwvn4s2o6Gsaq%2FPJapQQ0%2B%2BX2LsqL1tuthNeLjCnh7SqQC%2BmwHCAuN110hN5Yx6aweJxgwHO2amzf09pOdEIaeZgZRtNyXnErdSdI2HQqSc6depfMVN48xdtQ%3D%3D</v>
+      </c>
+      <c r="D111" t="str">
+        <v>R$ 135,41</v>
+      </c>
+      <c r="E111" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_626928-MLB82004918446_022025-O.webp</v>
+      </c>
+      <c r="F111" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Tira Manchas Percarbonato Calisul Brancas E Coloridas - 1kg</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C112" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BCKskL9L6XAML25sXtve8BP5UWhPeS9e%2BEnaMvD7vkW%2FAUmhUHQdgZxuFf7tGzVR8s1VzOJ2%2Bc%2B0hJVVuZfHrQkmB1RPdk5RvNEWbMNWHf4scjIv4eE2KR8DP6qmcBaKSaxfVadqX6GZSatkddDlApisBvtWhk%2FUMf8CRhQCj837Ti2zx9mwaxPzdabtE7kjIGSylQ%3D%3D</v>
+      </c>
+      <c r="D112" t="str">
+        <v>R$ 29,99</v>
+      </c>
+      <c r="E112" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_828760-MLB106129678450_022026-O.webp</v>
+      </c>
+      <c r="F112" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>Eudora Kit Presente Dia Das Mães Velvet Authentic</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C113" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BJUJiJf8mcktWj1rWfitSv3EKgRNai32uOPRqshoDQKW5gudiPWNcvjgdrpTSvcY8WA0Qsg%2BslXj75Zq5cgkdflnGD2JUJ5%2BA8%2BbTD8LtxXJh170wRp%2FAwBq%2FkgB2T%2BydkIVt3v4PGGshBQI2kLWsQL4aXU0A0YarAMzGXQu7gAGOhY1VSqIDMYOJ%2FXKI2kjXJkDps%2FFPrf8TxJ1ig%3D%3D</v>
+      </c>
+      <c r="D113" t="str">
+        <v>R$ 162,89</v>
+      </c>
+      <c r="E113" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_908328-MLB106403961018_022026-O.webp</v>
+      </c>
+      <c r="F113" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>Mini Compressor Digital Simake Bomba De Encher Pneus Portátil Para Carro Bicicleta Motocicletas Cor Preto Com Calibrador</v>
+      </c>
+      <c r="B114" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C114" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BE0BI6W9BrU%2FDMWGCSVElZqEai2BsYbCvv7Px8AbM1mMPlZXvd%2BASlXKIilPxIhF2Zvo4tKNviCaF8B7Ahi1VeCu0ErXgWu%2FQ9lKgPxTeiZSIA4ELr%2BPvrzoV8mRyqhCrAQJxXJ3g6Uq3ArYTAzV%2FArEgJbPyBn76JQEZg9J1%2B83r9qqGf6xCVI%2B8A8ZKQPU3h2%2B1A%3D%3D</v>
+      </c>
+      <c r="D114" t="str">
+        <v>R$ 109,99</v>
+      </c>
+      <c r="E114" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_900674-MLA100087555981_122025-O.webp</v>
+      </c>
+      <c r="F114" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>Máscara De Nutrição Para Cabelos Secos Kérastase Nutritive Masquintense | 200ml |</v>
+      </c>
+      <c r="B115" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C115" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BE1ilXCu70ox4ei%2FLB%2BGAOg0N1VVb%2FuEw%2FWWgiwjQ4vHUUGSJ2vVPD%2FcJVTR4jJeTJKboocdYdSoeKWrTOqyOPYcDpbc9xvfG5mRoV3lajkopSCcD2DfuWSbDz30x5EUhkRvDuFCk39WEDternN68S2mqfK%2B6VnDpClaV0ceUhOv1BzjXsstuWupNcnLeoV1mpWSesk%3D</v>
+      </c>
+      <c r="D115" t="str">
+        <v>R$ 399,90</v>
+      </c>
+      <c r="E115" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_627616-MLA99439270890_112025-O.webp</v>
+      </c>
+      <c r="F115" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>Capa Protetora Colchão Box Casal Padrão Matelado Impermeável</v>
+      </c>
+      <c r="B116" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C116" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BHOuhW4WgSH%2Fvl1Em38DnIJXx0zVmKnJ%2FfQkyvacW5OhEVCQ%2BIOplS0%2Bwmo8KzopzkKt2O11%2FTYcHEmloueHZm%2BePHoy7VMDC89FyDoQKlGfzSpXv%2BC4IPno7NIZsCAdBWi3u4HmWtb7OxydkUfku%2BEX9P3X7U0lh9bOBpD9He37EWRKB7hEtypDT1909JUnsMA9Fg%3D%3D</v>
+      </c>
+      <c r="D116" t="str">
+        <v>R$ 78,90</v>
+      </c>
+      <c r="E116" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_639258-MLB82839590542_032025-O.webp</v>
+      </c>
+      <c r="F116" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Calça Jeans Wide Leg Feminina Cintura Alta Sem Lycra Stillge</v>
+      </c>
+      <c r="B117" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C117" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BOHHhw6nZF1SLwkRqIBJYkQvuVdTFSeiPRMuJbH8qk7HiZIXjRznLl3ks6TQOVNL%2FxUDTzDay8lTY4WbcGoTFck8ap078Dl%2BnBgOrThCz%2Blh5FFxgUc%2FOCwIz6WZN5BQTbZFK6Ok%2BYWP4AIRFf3QmnG8LmF0HMFdlK8gHizIXlqzg9s2BS%2BQB9fPziZTO%2B4wB8uBfQ%3D%3D</v>
+      </c>
+      <c r="D117" t="str">
+        <v>R$ 109,99</v>
+      </c>
+      <c r="E117" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_717613-MLB96633630079_102025-O.webp</v>
+      </c>
+      <c r="F117" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>Kit Com 10 Caixa De Papelão Maleta Para Mudança De 50x40x30 Pardo Marrom-claro</v>
+      </c>
+      <c r="B118" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C118" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BCM%2F71rO2pw91rAzTealB4TBIqWDQJ6neDPH%2FGPXH5OFkgmZ3G3Xm77a0yqA1OKJAhFoQYLFY6v9ucXaj%2FanRmy92tFA5dUAP7uNlVIELALUc8E6oLKbAOkMPNFn%2BThZNIyQR6Dro5m427syUPBY6dQAmQtToEqYQasEuef1ibXVF%2BOMTJ5dztMfQUW98SUo6lh2qA%3D%3D</v>
+      </c>
+      <c r="D118" t="str">
+        <v>R$ 73,95</v>
+      </c>
+      <c r="E118" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_691630-MLA110062568687_042026-O.webp</v>
+      </c>
+      <c r="F118" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>Moletom Liso Algodão Unissex Blusa De Frio Canguru Flanelado G Preto</v>
+      </c>
+      <c r="B119" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C119" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BH7C3%2FJBo%2FICOjoXMxXBkFG%2B5MnB1D1T2kGd2Px926syrprmH44uqKhc8x4z1nzkg9306cvUIb4GbH89PACaq%2BI1cH3ZcGPfzieHSZfotkx3GLqDLXImbRMoYL%2Bc%2F5MmNkCpKXaR9aipjV5jYVaeEU743cauUFlj0yVj0TVmbe2EUAv%2BhmBDJeNb7TuoKk%2FCzpyQQuS4nP1psquBpA%3D%3D</v>
+      </c>
+      <c r="D119" t="str">
+        <v>R$ 78,90</v>
+      </c>
+      <c r="E119" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_820407-MLB80062120741_102024-O.webp</v>
+      </c>
+      <c r="F119" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>Copo Térmico Gigante 1,2l Inox Com Tampa E Inox Canudo</v>
+      </c>
+      <c r="B120" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C120" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BNs1yv%2FW3J%2FlbC2jd3z7WdNg6xfhy4vP%2B2yfZ0TWvZwolYO7D9hYYz7MOhmmm9jfvdHV11kXElNDG08eTkC4BD0YiShwOkgKoCUPWNhtspkMKBScV3pjLFnWTBYQ3Bx4qeAqwfa%2Bzri2iIrnDovc%2FWYZTHuo1Zm0NXXJvMNxMhm9fAiOk2DSYaDABYMWzHvL9KDhtw%3D%3D</v>
+      </c>
+      <c r="D120" t="str">
+        <v>R$ 99,98</v>
+      </c>
+      <c r="E120" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_637472-MLB111022989591_042026-O.webp</v>
+      </c>
+      <c r="F120" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>Copo Monster 500ml Com Alça - Kit Completo</v>
+      </c>
+      <c r="B121" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C121" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BK%2BM8OUzsTyj3EhxHIjRhJiDX1WurKD1HszLtIcti7Smkwv0oknu9ZMGILhifcKnEZUvBXVRup9PD73Eg1SHjgoYs8h2u7HXM19Uuz5kZgD7rDlylnRrbYeWQeMtOv%2FY8Br2vHidGcPr3NRKPxLBtgcdsc8OrMJ8TeOmnQMSWZzUPuGqtqpSJcqrce%2FxVQSQ%2FOnngg%3D%3D</v>
+      </c>
+      <c r="D121" t="str">
+        <v>R$ 79,90</v>
+      </c>
+      <c r="E121" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_882790-MLB110606211421_042026-O.webp</v>
+      </c>
+      <c r="F121" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>Camisa Social Masculina Slim Premium Manga Longa / Curta</v>
+      </c>
+      <c r="B122" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C122" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BAU6Zn1PHf4f2Jq42aQ1pWulEIX7qFZ754uFdWYq310qMX9ILXLDj9Ezi%2FGlfEkJ%2B99CclP7fWACASFTeorI0Uf9J2zwklCzof7sc8FlyR482DG8bZL9tv77v9jzXLPLsfTbIJL0v5Viqp8OJhY352vYVqKYVRCN1HAU6v0pEsBZaOBvkFSBtPgXErwWCo1g%2BHQC3Q%3D%3D</v>
+      </c>
+      <c r="D122" t="str">
+        <v>R$ 69,90</v>
+      </c>
+      <c r="E122" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_864582-MLB108696083701_032026-O.webp</v>
+      </c>
+      <c r="F122" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>Apoio Para Pés Ergonômico Multivisão Apoio-pr Apoiador Com Regulagem Escritório</v>
+      </c>
+      <c r="B123" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C123" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BAcYBVC%2Frl%2Be9QBpptBaPLjSLp5Z1JKYadIiTVKF04H65MSPLIDu43dM8ZOH3ioDGG2TgoYKXJJSMhOiCfsaswxlt9yuyqL5rgaXM7QANNCy0tqnyJBJIKnUO6as4d0s8CtxjCNTJcaqhgyOC6Sy%2BHi%2FUgZRNvyfOK2o9NlPR6vsEwHuBEsWEtg%2BPqjJmP9gZIcUTg%3D%3D</v>
+      </c>
+      <c r="D123" t="str">
+        <v>R$ 59,75</v>
+      </c>
+      <c r="E123" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_775703-MLA96130701933_102025-O.webp</v>
+      </c>
+      <c r="F123" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>Patinete Infantil 3 Rodas Dobrável Com Led Conect Brinq Bv0011 Brinquedo Para Crianças Estável, Seguro E Divertido Colorido Azul</v>
+      </c>
+      <c r="B124" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C124" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BHfhK8o2%2BecjWhKVBV4ZlS9Vh5d5JfVPVKOCjZ0qyZCz7PSaFr2ebCuHnnHRF3uW0KKgN00ZZVKi8k3rUbUsx1Jc7Uzu9ToWDgg4%2FYS95rMvBO0vcy3DCKf4C0EzuVPOSuSt4tBAIcV4w3NeqI%2B58jtvx3eeVN6ug8yaG5eaN4Ke%2Bkcp8OXyNUwk5QlOFzkd7pncAw%3D%3D</v>
+      </c>
+      <c r="D124" t="str">
+        <v>R$ 199,90</v>
+      </c>
+      <c r="E124" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_647379-MLA100478895706_122025-O.webp</v>
+      </c>
+      <c r="F124" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>Eudora Imensi Kit (2 Produtos)</v>
+      </c>
+      <c r="B125" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C125" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BJCA6ROWog9bsrnDqISVcWvndD%2FMNT1G%2Ft5RDVK%2FsxLZGlf5%2FEFUFrSGA33lg1eOI5P9pXFVg6ZkLy8UPlfDR1iC9yaYhWYwe0xuLsy%2Bul12jbH7RLVYN3f5%2BpfjqfQVV19AxG6KlaXM%2F7WE1cb%2BMmTJTJfnP3YVoeFmcxd9ep58Lpq5D0vPq%2BG1ZjkUSYaACgPulFgQvAsDYs3juQ%3D%3D</v>
+      </c>
+      <c r="D125" t="str">
+        <v>R$ 202,89</v>
+      </c>
+      <c r="E125" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_731387-MLB106473367680_022026-O.webp</v>
+      </c>
+      <c r="F125" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>Kit 4 Potes Acrílico 3,8l Organizador Geladeira Rebirth</v>
+      </c>
+      <c r="B126" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C126" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BO%2FXCp6hJ1pMjI8owt3JmzTVo%2B6Cq9Xjmz3Er%2Bj0TWPG5hnhn2MlhU5YbRnCitxOqi5z3pQxjHZTipCUdj3lZ3A1KDDV0sHgK%2FlIYkgjXuJDzoZA0GeN52ED44DZP6vTQo1iCl4aSUhVVv4bmKuTknAC895jQuV8U3gkb7aUuCObonxYW58tlVzzBiGCSyNCZlznrw%3D%3D</v>
+      </c>
+      <c r="D126" t="str">
+        <v>R$ 199,90</v>
+      </c>
+      <c r="E126" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_735971-MLA95941810245_102025-O.webp</v>
+      </c>
+      <c r="F126" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>Varal De Chão Grande De Roupas 3 Andares Dobrável Cor Azul Kontuz 170 Cm</v>
+      </c>
+      <c r="B127" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C127" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BIg13bLHyL%2Bijbn3MWscIyivE1JD%2FlXdg4iL7mLYr75QjDy1Hl1JD8UGIiG%2BH9k9rFlNxPPpXVCiTYcGtdN5VlFKGdwfOU67%2BedmXqyQdYeEfmN%2FX1hL5Uht5BtA9YNTOuxZcpJVAweSqIokpuiwNeU4aXQ7u9BlCnhpZJAHiqrXn7jTLNfBAs1yHDIzjZABEp71Ag%3D%3D</v>
+      </c>
+      <c r="D127" t="str">
+        <v>R$ 119,90</v>
+      </c>
+      <c r="E127" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_712866-MLA109482654866_042026-O.webp</v>
+      </c>
+      <c r="F127" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>Kit C/ 4 Toalha De Banho Gigante 80 X 1,50 Atacado + Brinde Softmax</v>
+      </c>
+      <c r="B128" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C128" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BPe1cLMr284BLCVTKfJf1IH9xdauseaZpVqWsGPbyYpRBQDV08Ad%2BJHvTwfY2TBREJ8F%2By%2Fgzwn0u%2FBPTgKhWSMQknMdVh8qAMD%2FaFTJy7X%2BgAUJJqv3j40YTRoTJFsC1PGgNpc0CE06yarrs1s610tPPw6V5vcQvoSeP3N75F6ES4YnDuNEVI8HBOLMA491PKkbrQ%3D%3D</v>
+      </c>
+      <c r="D128" t="str">
+        <v>R$ 154,22</v>
+      </c>
+      <c r="E128" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_957812-MLB95817097996_102025-O.webp</v>
+      </c>
+      <c r="F128" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>Torneira Para Cozinha Dazie Metais Com Filtro Bancada Flexível Em Abs Cromado</v>
+      </c>
+      <c r="B129" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C129" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BFjCvY3SrWrUhrFPMI5lq%2FM1%2FDpxgtIByWm9KIjHm%2BgTl%2B00DQ7pUjA2fO2Sddf1ZWQzaTaR2POc5TXwfArnn%2BxbcNdpFMb1EJA3O%2FetaMxcRfLGT1QH%2F3MwwogWDUlOULsDoSJoBozOVj4bLsLd7oINhuRo63clz3CB0OpJ1DU2S0xtsOj9uT9tzlDPkRrW30h9OQ%3D%3D</v>
+      </c>
+      <c r="D129" t="str">
+        <v>R$ 108,62</v>
+      </c>
+      <c r="E129" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_734158-MLA100001103325_112025-O.webp</v>
+      </c>
+      <c r="F129" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>Calça Mom Jeans Feminina Cintura Alta Marmorizada</v>
+      </c>
+      <c r="B130" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C130" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BLUureWWHHVafaRNYf2I15foiVIwDDFYgUJjhhHQjHV8YxeWhIS6AGKWKbufHI%2BfA7VA8D0ltjiYPW%2FPlZ0VI0GJMGAIKjxWRG5sLV4n1xFvr6rU41ifsWlPMsd8o53RAEoGvBpYDaSbJaiMaP%2BaxYERhhgggjIVlEd2TaCagD5QiwzQvbLujUo3UtB7XGIRXXGWrA%3D%3D</v>
+      </c>
+      <c r="D130" t="str">
+        <v>R$ 99,99</v>
+      </c>
+      <c r="E130" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_799787-MLB85664619217_062025-O.webp</v>
+      </c>
+      <c r="F130" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>Martelete Perfurador Rompedor Professional 26mm 1300w Sds</v>
+      </c>
+      <c r="B131" t="str">
+        <v>Oferta Especial Mercado Livre</v>
+      </c>
+      <c r="C131" t="str">
+        <v>https://www.mercadolivre.com.br/social/ab20260421171952?matt_word=ab20260421171952&amp;matt_tool=50857810&amp;forceInApp=true&amp;ref=BIABz2Z%2F3g%2FG%2FF9KyMrD7mjine1OlOtqh1fYk4c9usb3uPJqrP6PIGlznA2O88Q4dWG5ZYH2OuzlRNeUKJFBqY8U40QIBmlhb8%2FbM1UYpaTum5NtjUhII46wdmY7WX9A5REemdDoWXES9Q3uBXgjdhMnzhalgkBKTBGUtLZn7kAdLH6YR8ph4ACxOVW%2F0AJWbQKFog%3D%3D</v>
+      </c>
+      <c r="D131" t="str">
+        <v>R$ 443,16</v>
+      </c>
+      <c r="E131" t="str">
+        <v>https://http2.mlstatic.com/D_NQ_NP_973130-MLB80836312140_122024-O.webp</v>
+      </c>
+      <c r="F131" t="str">
+        <v>Mercado Livre</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F131"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>